<commit_message>
Use mask seeds 42-44 and 40% masking level; masking figure for seed 42 only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XQmcR8UJ8WPn3HMfEePqkv
</commit_message>
<xml_diff>
--- a/results/paper/paper_assets.xlsx
+++ b/results/paper/paper_assets.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="207">
   <si>
     <t>Well</t>
   </si>
@@ -150,16 +150,16 @@
     <t>3</t>
   </si>
   <si>
-    <t>39.7 ± 0.1</t>
-  </si>
-  <si>
-    <t>34.9 ± 0.1</t>
-  </si>
-  <si>
-    <t>21.1 ± 0.0</t>
-  </si>
-  <si>
-    <t>4.3 ± 0.1</t>
+    <t>30.2 ± 0.1</t>
+  </si>
+  <si>
+    <t>30.1 ± 0.1</t>
+  </si>
+  <si>
+    <t>29.1 ± 0.0</t>
+  </si>
+  <si>
+    <t>10.6 ± 0.0</t>
   </si>
   <si>
     <t>Masked cells per seed</t>
@@ -168,7 +168,7 @@
     <t>Share of rows (%)</t>
   </si>
   <si>
-    <t>2043 ± 0</t>
+    <t>2725 ± 0</t>
   </si>
   <si>
     <t>Method</t>
@@ -195,472 +195,454 @@
     <t>LGBM</t>
   </si>
   <si>
-    <t>108.7 ± 5.1</t>
-  </si>
-  <si>
-    <t>131.2 ± 4.3</t>
-  </si>
-  <si>
-    <t>88.6 ± 5.3</t>
-  </si>
-  <si>
-    <t>10.55 ± 0.08</t>
-  </si>
-  <si>
-    <t>7.02 ± 0.14</t>
-  </si>
-  <si>
-    <t>6.43 ± 0.26</t>
-  </si>
-  <si>
-    <t>0.145 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.115 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.111 ± 0.004</t>
-  </si>
-  <si>
-    <t>27.1 ± 0.3</t>
-  </si>
-  <si>
-    <t>25.9 ± 0.9</t>
-  </si>
-  <si>
-    <t>14.6 ± 0.5</t>
-  </si>
-  <si>
-    <t>8.71 ± 0.10</t>
-  </si>
-  <si>
-    <t>5.04 ± 0.09</t>
-  </si>
-  <si>
-    <t>4.51 ± 0.14</t>
+    <t>110.9 ± 0.1</t>
+  </si>
+  <si>
+    <t>103.3 ± 0.7</t>
+  </si>
+  <si>
+    <t>97.9 ± 0.3</t>
+  </si>
+  <si>
+    <t>10.57 ± 0.01</t>
+  </si>
+  <si>
+    <t>7.10 ± 0.02</t>
+  </si>
+  <si>
+    <t>6.68 ± 0.09</t>
+  </si>
+  <si>
+    <t>0.148 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.118 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.124 ± 0.000</t>
+  </si>
+  <si>
+    <t>27.6 ± 0.1</t>
+  </si>
+  <si>
+    <t>21.3 ± 0.4</t>
+  </si>
+  <si>
+    <t>17.7 ± 0.2</t>
+  </si>
+  <si>
+    <t>8.76 ± 0.00</t>
+  </si>
+  <si>
+    <t>5.05 ± 0.02</t>
+  </si>
+  <si>
+    <t>4.85 ± 0.06</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.083 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.063 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.058 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.055 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.157 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.105 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.099 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.086 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.069 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.072 ± 0.000</t>
+  </si>
+  <si>
+    <t>-0.05 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.09 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.18 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.53 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.58 ± 0.01</t>
+  </si>
+  <si>
+    <t>-0.09 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.31 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.24 ± 0.00</t>
+  </si>
+  <si>
+    <t>k=1</t>
+  </si>
+  <si>
+    <t>k=2</t>
+  </si>
+  <si>
+    <t>k=3</t>
+  </si>
+  <si>
+    <t>0.094 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.068 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.099 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.072 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.113 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.087 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.085 ± 0.001</t>
+  </si>
+  <si>
+    <t>R2 wells min</t>
+  </si>
+  <si>
+    <t>R2 wells max</t>
+  </si>
+  <si>
+    <t>R2 sd across wells</t>
+  </si>
+  <si>
+    <t>Worst well</t>
+  </si>
+  <si>
+    <t>nRMSE sd across wells</t>
+  </si>
+  <si>
+    <t>nRMSE sd across seeds</t>
+  </si>
+  <si>
+    <t>max nRMSE sd across seeds (per well)</t>
+  </si>
+  <si>
+    <t>0.112 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.089 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.077 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.058 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.025 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.155 ± 0.003</t>
   </si>
   <si>
     <t>0.116 ± 0.001</t>
   </si>
   <si>
-    <t>0.071 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.070 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.062 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.074 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.050 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.157 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.104 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.095 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.085 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.067 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.065 ± 0.002</t>
-  </si>
-  <si>
-    <t>-0.05 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.55 ± 0.24</t>
-  </si>
-  <si>
-    <t>0.30 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.53 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.61 ± 0.04</t>
-  </si>
-  <si>
-    <t>-0.08 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.32 ± 0.05</t>
-  </si>
-  <si>
-    <t>0.37 ± 0.02</t>
-  </si>
-  <si>
-    <t>k=1</t>
-  </si>
-  <si>
-    <t>k=2</t>
-  </si>
-  <si>
-    <t>k=3</t>
-  </si>
-  <si>
-    <t>0.095 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.078 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.064 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.100 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.081 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.070 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.115 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.092 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.080 ± 0.002</t>
-  </si>
-  <si>
-    <t>R2 wells min</t>
-  </si>
-  <si>
-    <t>R2 wells max</t>
-  </si>
-  <si>
-    <t>R2 sd across wells</t>
-  </si>
-  <si>
-    <t>Worst well</t>
-  </si>
-  <si>
-    <t>nRMSE sd across wells</t>
-  </si>
-  <si>
-    <t>nRMSE sd across seeds</t>
-  </si>
-  <si>
-    <t>max nRMSE sd across seeds (per well)</t>
-  </si>
-  <si>
-    <t>0.104 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.078 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.069 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.051 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.013 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.138 ± 0.008</t>
-  </si>
-  <si>
-    <t>0.107 ± 0.010</t>
-  </si>
-  <si>
-    <t>0.084 ± 0.010</t>
-  </si>
-  <si>
-    <t>0.123 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.083 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.089 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.077 ± 0.009</t>
-  </si>
-  <si>
-    <t>0.040 ± 0.002</t>
+    <t>0.091 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.131 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.094 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.093 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.060 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.048 ± 0.001</t>
   </si>
   <si>
     <t>0.000 ± 0.000</t>
   </si>
   <si>
-    <t>0.154 ± 0.017</t>
-  </si>
-  <si>
-    <t>0.071 ± 0.013</t>
-  </si>
-  <si>
-    <t>0.014 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.128 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.073 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.079 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.059 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.060 ± 0.031</t>
-  </si>
-  <si>
-    <t>0.154 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.109 ± 0.010</t>
-  </si>
-  <si>
-    <t>0.098 ± 0.012</t>
-  </si>
-  <si>
-    <t>0.135 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.114 ± 0.025</t>
-  </si>
-  <si>
-    <t>0.069 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.040 ± 0.003</t>
+    <t>0.160 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.081 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.007 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.138 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.080 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.054 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.022 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.158 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.112 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.098 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.138 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.089 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.092 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.059 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.043 ± 0.000</t>
   </si>
   <si>
     <t>0.001 ± 0.000</t>
   </si>
   <si>
-    <t>0.156 ± 0.024</t>
-  </si>
-  <si>
-    <t>0.073 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.137 ± 0.051</t>
-  </si>
-  <si>
-    <t>0.178 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.102 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.098 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.132 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.068 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.031 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.217 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.118 ± 0.008</t>
-  </si>
-  <si>
-    <t>0.102 ± 0.012</t>
-  </si>
-  <si>
-    <t>0.200 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.103 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.099 ± 0.008</t>
-  </si>
-  <si>
-    <t>0.120 ± 0.002</t>
+    <t>0.164 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.072 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.037 ± 0.015</t>
+  </si>
+  <si>
+    <t>0.179 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.103 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.102 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.133 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.032 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.217 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.122 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.199 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.107 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.101 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.120 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.000</t>
   </si>
   <si>
     <t>0.003 ± 0.000</t>
   </si>
   <si>
-    <t>0.178 ± 0.009</t>
-  </si>
-  <si>
-    <t>0.075 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.013 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.64 ± 0.04</t>
-  </si>
-  <si>
-    <t>-0.01 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.26 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.70 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.44 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.82 ± 0.09</t>
-  </si>
-  <si>
-    <t>0.58 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.18 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.24 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.54 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.23 ± 0.02</t>
+    <t>0.183 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.078 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.014 ± 0.000</t>
+  </si>
+  <si>
+    <t>-0.24 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.11 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.63 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.27 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.38 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.48 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.10 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.12 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.11 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.06 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.65 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.32 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.97 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.23 ± 0.03</t>
+  </si>
+  <si>
+    <t>-0.07 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.69 ± 0.06</t>
+  </si>
+  <si>
+    <t>0.35 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.21 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.60 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.37 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.53 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.46 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.15 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.04 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.42 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.21 ± 0.00</t>
   </si>
   <si>
     <t>0.08 ± 0.01</t>
   </si>
   <si>
-    <t>0.42 ± 0.15</t>
-  </si>
-  <si>
-    <t>0.50 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.94 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.25 ± 0.09</t>
-  </si>
-  <si>
-    <t>0.09 ± 0.23</t>
-  </si>
-  <si>
-    <t>-0.49 ± 0.54</t>
-  </si>
-  <si>
-    <t>0.45 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.07 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.60 ± 0.06</t>
-  </si>
-  <si>
-    <t>0.24 ± 0.16</t>
-  </si>
-  <si>
-    <t>-3.30 ± 3.81</t>
-  </si>
-  <si>
-    <t>0.48 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.15 ± 0.05</t>
-  </si>
-  <si>
-    <t>-0.03 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.45 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.29 ± 0.03</t>
-  </si>
-  <si>
-    <t>-0.50 ± 0.52</t>
-  </si>
-  <si>
-    <t>0.54 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.51 ± 0.06</t>
-  </si>
-  <si>
-    <t>0.30 ± 0.12</t>
-  </si>
-  <si>
-    <t>0.22 ± 0.15</t>
-  </si>
-  <si>
-    <t>0.03 ± 0.04</t>
-  </si>
-  <si>
-    <t>-144.32 ± 76.08</t>
-  </si>
-  <si>
-    <t>-0.06 ± 0.01</t>
-  </si>
-  <si>
-    <t>-1.11 ± 0.08</t>
-  </si>
-  <si>
-    <t>-0.16 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.09 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.02 ± 0.01</t>
+    <t>0.66 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.41 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.19 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.16 ± 0.04</t>
+  </si>
+  <si>
+    <t>-9.39 ± 8.61</t>
+  </si>
+  <si>
+    <t>-0.08 ± 0.00</t>
+  </si>
+  <si>
+    <t>-1.06 ± 0.01</t>
+  </si>
+  <si>
+    <t>-0.16 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.10 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.02 ± 0.00</t>
   </si>
   <si>
     <t>-0.03 ± 0.00</t>
   </si>
   <si>
-    <t>-0.04 ± 0.02</t>
-  </si>
-  <si>
     <t>-0.00 ± 0.00</t>
   </si>
   <si>
-    <t>-0.13 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.21 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.17 ± 0.03</t>
-  </si>
-  <si>
-    <t>-0.13 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.39 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.44 ± 0.02</t>
-  </si>
-  <si>
-    <t>-1.57 ± 0.65</t>
-  </si>
-  <si>
-    <t>-0.01 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.22 ± 0.02</t>
+    <t>-0.13 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.20 ± 0.01</t>
+  </si>
+  <si>
+    <t>-0.14 ± 0.01</t>
+  </si>
+  <si>
+    <t>-0.40 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.48 ± 0.00</t>
+  </si>
+  <si>
+    <t>-1.04 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.01 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.22 ± 0.00</t>
   </si>
 </sst>
 </file>
@@ -1596,7 +1578,7 @@
         <v>42</v>
       </c>
       <c r="C2">
-        <v>34.3</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1607,7 +1589,7 @@
         <v>43</v>
       </c>
       <c r="C3">
-        <v>44.1</v>
+        <v>43.2</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1618,7 +1600,7 @@
         <v>44</v>
       </c>
       <c r="C4">
-        <v>18.9</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1629,7 +1611,7 @@
         <v>45</v>
       </c>
       <c r="C5">
-        <v>2.7</v>
+        <v>6.4</v>
       </c>
     </row>
   </sheetData>
@@ -1661,7 +1643,7 @@
         <v>48</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1672,7 +1654,7 @@
         <v>48</v>
       </c>
       <c r="C3">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1683,7 +1665,7 @@
         <v>48</v>
       </c>
       <c r="C4">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1730,10 +1712,10 @@
         <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1750,10 +1732,10 @@
         <v>67</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1770,10 +1752,10 @@
         <v>68</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1790,10 +1772,10 @@
         <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1810,10 +1792,10 @@
         <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1830,10 +1812,10 @@
         <v>71</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1847,13 +1829,13 @@
         <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1867,13 +1849,13 @@
         <v>64</v>
       </c>
       <c r="D9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1887,13 +1869,13 @@
         <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1911,13 +1893,13 @@
         <v>49</v>
       </c>
       <c r="B1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
-      </c>
-      <c r="D1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1925,13 +1907,13 @@
         <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1939,13 +1921,13 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1953,13 +1935,13 @@
         <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1980,25 +1962,25 @@
         <v>49</v>
       </c>
       <c r="C1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" t="s">
         <v>104</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>105</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>106</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>107</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>108</v>
-      </c>
-      <c r="H1" t="s">
-        <v>109</v>
-      </c>
-      <c r="I1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -2009,25 +1991,25 @@
         <v>54</v>
       </c>
       <c r="C2">
-        <v>-1.57</v>
+        <v>-1.04</v>
       </c>
       <c r="D2">
         <v>-0.03</v>
       </c>
       <c r="E2">
-        <v>0.59</v>
+        <v>0.37</v>
       </c>
       <c r="F2" t="s">
         <v>13</v>
       </c>
       <c r="G2">
-        <v>0.047</v>
+        <v>0.048</v>
       </c>
       <c r="H2">
-        <v>0.0029</v>
+        <v>0.0001</v>
       </c>
       <c r="I2">
-        <v>0.0122</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2038,25 +2020,25 @@
         <v>55</v>
       </c>
       <c r="C3">
-        <v>-144.32</v>
+        <v>-9.390000000000001</v>
       </c>
       <c r="D3">
-        <v>0.3</v>
+        <v>0.53</v>
       </c>
       <c r="E3">
-        <v>58.64</v>
+        <v>3.91</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
       </c>
       <c r="G3">
-        <v>0.048</v>
+        <v>0.043</v>
       </c>
       <c r="H3">
-        <v>0.0025</v>
+        <v>0.0004</v>
       </c>
       <c r="I3">
-        <v>0.0506</v>
+        <v>0.0155</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2067,25 +2049,25 @@
         <v>56</v>
       </c>
       <c r="C4">
-        <v>-0.49</v>
+        <v>0.06</v>
       </c>
       <c r="D4">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="E4">
-        <v>0.52</v>
+        <v>0.37</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>0.041</v>
+        <v>0.045</v>
       </c>
       <c r="H4">
-        <v>0.003</v>
+        <v>0.0002</v>
       </c>
       <c r="I4">
-        <v>0.0103</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2096,13 +2078,13 @@
         <v>54</v>
       </c>
       <c r="C5">
-        <v>-0.39</v>
+        <v>-0.4</v>
       </c>
       <c r="D5">
         <v>-0.01</v>
       </c>
       <c r="E5">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F5" t="s">
         <v>13</v>
@@ -2111,10 +2093,10 @@
         <v>0.038</v>
       </c>
       <c r="H5">
-        <v>0.0012</v>
+        <v>0.0001</v>
       </c>
       <c r="I5">
-        <v>0.009299999999999999</v>
+        <v>0.0038</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2125,25 +2107,25 @@
         <v>55</v>
       </c>
       <c r="C6">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="D6">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="E6">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
       </c>
       <c r="G6">
-        <v>0.037</v>
+        <v>0.043</v>
       </c>
       <c r="H6">
-        <v>0.002</v>
+        <v>0.0003</v>
       </c>
       <c r="I6">
-        <v>0.0242</v>
+        <v>0.0027</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2154,10 +2136,10 @@
         <v>56</v>
       </c>
       <c r="C7">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="D7">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="E7">
         <v>0.16</v>
@@ -2166,13 +2148,13 @@
         <v>14</v>
       </c>
       <c r="G7">
-        <v>0.034</v>
+        <v>0.041</v>
       </c>
       <c r="H7">
-        <v>0.0038</v>
+        <v>0.0013</v>
       </c>
       <c r="I7">
-        <v>0.0172</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2183,25 +2165,25 @@
         <v>54</v>
       </c>
       <c r="C8">
-        <v>-1.11</v>
+        <v>-1.06</v>
       </c>
       <c r="D8">
         <v>-0</v>
       </c>
       <c r="E8">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
       </c>
       <c r="G8">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
       <c r="H8">
-        <v>0.0017</v>
+        <v>0.0001</v>
       </c>
       <c r="I8">
-        <v>0.0076</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2212,25 +2194,25 @@
         <v>55</v>
       </c>
       <c r="C9">
-        <v>-0.07000000000000001</v>
+        <v>-0.21</v>
       </c>
       <c r="D9">
-        <v>0.51</v>
+        <v>0.46</v>
       </c>
       <c r="E9">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
       </c>
       <c r="G9">
-        <v>0.023</v>
+        <v>0.025</v>
       </c>
       <c r="H9">
-        <v>0.0041</v>
+        <v>0.0001</v>
       </c>
       <c r="I9">
-        <v>0.0104</v>
+        <v>0.0019</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2241,13 +2223,13 @@
         <v>56</v>
       </c>
       <c r="C10">
-        <v>-0.01</v>
+        <v>-0.24</v>
       </c>
       <c r="D10">
-        <v>0.5</v>
+        <v>0.32</v>
       </c>
       <c r="E10">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -2256,10 +2238,10 @@
         <v>0.024</v>
       </c>
       <c r="H10">
-        <v>0.0024</v>
+        <v>0.0002</v>
       </c>
       <c r="I10">
-        <v>0.0134</v>
+        <v>0.0015</v>
       </c>
     </row>
   </sheetData>
@@ -2300,10 +2282,10 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E2" t="s">
-        <v>161</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2317,10 +2299,10 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2334,10 +2316,10 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2351,10 +2333,10 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2368,10 +2350,10 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2385,10 +2367,10 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2402,10 +2384,10 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2419,10 +2401,10 @@
         <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2436,10 +2418,10 @@
         <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2453,10 +2435,10 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E11" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2470,10 +2452,10 @@
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E12" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2487,10 +2469,10 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E13" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2504,10 +2486,10 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E14" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2521,10 +2503,10 @@
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E15" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -2538,10 +2520,10 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E16" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2555,10 +2537,10 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E17" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2572,10 +2554,10 @@
         <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2589,10 +2571,10 @@
         <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E19" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2606,10 +2588,10 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E20" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2623,10 +2605,10 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2640,10 +2622,10 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="E22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2657,10 +2639,10 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E23" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -2674,10 +2656,10 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E24" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -2691,10 +2673,10 @@
         <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E25" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -2708,10 +2690,10 @@
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E26" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -2725,10 +2707,10 @@
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E27" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2742,10 +2724,10 @@
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E28" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2759,10 +2741,10 @@
         <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E29" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2776,10 +2758,10 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="E30" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2796,7 +2778,7 @@
         <v>137</v>
       </c>
       <c r="E31" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2813,7 +2795,7 @@
         <v>138</v>
       </c>
       <c r="E32" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -2830,7 +2812,7 @@
         <v>139</v>
       </c>
       <c r="E33" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2847,7 +2829,7 @@
         <v>140</v>
       </c>
       <c r="E34" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -2864,7 +2846,7 @@
         <v>141</v>
       </c>
       <c r="E35" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2881,7 +2863,7 @@
         <v>142</v>
       </c>
       <c r="E36" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -2898,7 +2880,7 @@
         <v>143</v>
       </c>
       <c r="E37" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2915,7 +2897,7 @@
         <v>144</v>
       </c>
       <c r="E38" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2932,7 +2914,7 @@
         <v>145</v>
       </c>
       <c r="E39" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2949,7 +2931,7 @@
         <v>146</v>
       </c>
       <c r="E40" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -2966,7 +2948,7 @@
         <v>147</v>
       </c>
       <c r="E41" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2980,10 +2962,10 @@
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>148</v>
+        <v>81</v>
       </c>
       <c r="E42" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2997,10 +2979,10 @@
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E43" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -3014,10 +2996,10 @@
         <v>11</v>
       </c>
       <c r="D44" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E44" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3031,10 +3013,10 @@
         <v>11</v>
       </c>
       <c r="D45" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E45" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -3048,10 +3030,10 @@
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="E46" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -3065,10 +3047,10 @@
         <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E47" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3082,10 +3064,10 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E48" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -3099,10 +3081,10 @@
         <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E49" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -3116,10 +3098,10 @@
         <v>13</v>
       </c>
       <c r="D50" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E50" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -3133,10 +3115,10 @@
         <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E51" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3150,10 +3132,10 @@
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E52" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3167,10 +3149,10 @@
         <v>14</v>
       </c>
       <c r="D53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E53" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3184,10 +3166,10 @@
         <v>14</v>
       </c>
       <c r="D54" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E54" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3201,10 +3183,10 @@
         <v>14</v>
       </c>
       <c r="D55" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E55" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert masking level to 30%; plot only the first seed (42)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XQmcR8UJ8WPn3HMfEePqkv
</commit_message>
<xml_diff>
--- a/results/paper/paper_assets.xlsx
+++ b/results/paper/paper_assets.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="212">
   <si>
     <t>Well</t>
   </si>
@@ -150,16 +150,16 @@
     <t>3</t>
   </si>
   <si>
-    <t>30.2 ± 0.1</t>
-  </si>
-  <si>
-    <t>30.1 ± 0.1</t>
-  </si>
-  <si>
-    <t>29.1 ± 0.0</t>
-  </si>
-  <si>
-    <t>10.6 ± 0.0</t>
+    <t>40.0 ± 0.1</t>
+  </si>
+  <si>
+    <t>34.6 ± 0.3</t>
+  </si>
+  <si>
+    <t>20.8 ± 0.1</t>
+  </si>
+  <si>
+    <t>4.6 ± 0.0</t>
   </si>
   <si>
     <t>Masked cells per seed</t>
@@ -168,7 +168,7 @@
     <t>Share of rows (%)</t>
   </si>
   <si>
-    <t>2725 ± 0</t>
+    <t>2043 ± 0</t>
   </si>
   <si>
     <t>Method</t>
@@ -195,106 +195,112 @@
     <t>LGBM</t>
   </si>
   <si>
-    <t>110.9 ± 0.1</t>
-  </si>
-  <si>
-    <t>103.3 ± 0.7</t>
-  </si>
-  <si>
-    <t>97.9 ± 0.3</t>
-  </si>
-  <si>
-    <t>10.57 ± 0.01</t>
-  </si>
-  <si>
-    <t>7.10 ± 0.02</t>
-  </si>
-  <si>
-    <t>6.68 ± 0.09</t>
-  </si>
-  <si>
-    <t>0.148 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.118 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.124 ± 0.000</t>
-  </si>
-  <si>
-    <t>27.6 ± 0.1</t>
-  </si>
-  <si>
-    <t>21.3 ± 0.4</t>
-  </si>
-  <si>
-    <t>17.7 ± 0.2</t>
-  </si>
-  <si>
-    <t>8.76 ± 0.00</t>
-  </si>
-  <si>
-    <t>5.05 ± 0.02</t>
-  </si>
-  <si>
-    <t>4.85 ± 0.06</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.083 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.063 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.058 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.055 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.157 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.105 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.099 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.086 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.069 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.072 ± 0.000</t>
+    <t>103.8 ± 3.2</t>
+  </si>
+  <si>
+    <t>129.7 ± 11.2</t>
+  </si>
+  <si>
+    <t>82.7 ± 4.5</t>
+  </si>
+  <si>
+    <t>10.55 ± 0.07</t>
+  </si>
+  <si>
+    <t>6.95 ± 0.15</t>
+  </si>
+  <si>
+    <t>6.34 ± 0.19</t>
+  </si>
+  <si>
+    <t>0.146 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.116 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.113 ± 0.001</t>
+  </si>
+  <si>
+    <t>26.7 ± 0.7</t>
+  </si>
+  <si>
+    <t>26.1 ± 1.7</t>
+  </si>
+  <si>
+    <t>13.9 ± 0.9</t>
+  </si>
+  <si>
+    <t>8.74 ± 0.04</t>
+  </si>
+  <si>
+    <t>4.99 ± 0.05</t>
+  </si>
+  <si>
+    <t>4.44 ± 0.15</t>
+  </si>
+  <si>
+    <t>0.117 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.072 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.059 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.073 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.047 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.157 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.103 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.094 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.085 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.067 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.066 ± 0.001</t>
+  </si>
+  <si>
+    <t>-0.06 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.65 ± 0.21</t>
+  </si>
+  <si>
+    <t>0.33 ± 0.04</t>
   </si>
   <si>
     <t>-0.05 ± 0.00</t>
   </si>
   <si>
-    <t>0.09 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.18 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.53 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.58 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.09 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.31 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.24 ± 0.00</t>
+    <t>0.54 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.62 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.08 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.32 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.35 ± 0.00</t>
   </si>
   <si>
     <t>k=1</t>
@@ -306,28 +312,31 @@
     <t>k=3</t>
   </si>
   <si>
-    <t>0.094 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.068 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.099 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.074 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.072 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.113 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.087 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.085 ± 0.001</t>
+    <t>0.092 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.060 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.100 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.114 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.091 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.078 ± 0.003</t>
   </si>
   <si>
     <t>R2 wells min</t>
@@ -351,298 +360,304 @@
     <t>max nRMSE sd across seeds (per well)</t>
   </si>
   <si>
-    <t>0.112 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.079 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.089 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.077 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.058 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.025 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.155 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.116 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.091 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.131 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.094 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.093 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.060 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.048 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.000 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.160 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.081 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.007 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.138 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.079 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.080 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.054 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.022 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.158 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.112 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.098 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.138 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.089 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.092 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.059 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.043 ± 0.000</t>
+    <t>0.102 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.083 ± 0.011</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.051 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.010 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.140 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.106 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.117 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.008</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.010</t>
+  </si>
+  <si>
+    <t>0.039 ± 0.003</t>
   </si>
   <si>
     <t>0.001 ± 0.000</t>
   </si>
   <si>
-    <t>0.164 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.072 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.037 ± 0.015</t>
-  </si>
-  <si>
-    <t>0.179 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.103 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.102 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.133 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.032 ± 0.000</t>
+    <t>0.150 ± 0.013</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.017 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.128 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.100 ± 0.009</t>
+  </si>
+  <si>
+    <t>0.080 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.057 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.022</t>
+  </si>
+  <si>
+    <t>0.151 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.107 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.090 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.130 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.086 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.093 ± 0.018</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.041 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.159 ± 0.014</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.092 ± 0.086</t>
+  </si>
+  <si>
+    <t>0.180 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.103 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.104 ± 0.008</t>
+  </si>
+  <si>
+    <t>0.132 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.069 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.031 ± 0.001</t>
   </si>
   <si>
     <t>0.217 ± 0.001</t>
   </si>
   <si>
-    <t>0.122 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.199 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.107 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.101 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.120 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.071 ± 0.000</t>
+    <t>0.117 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.094 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.197 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.109 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.085 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.120 ± 0.001</t>
   </si>
   <si>
     <t>0.003 ± 0.000</t>
   </si>
   <si>
-    <t>0.183 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.078 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.014 ± 0.000</t>
-  </si>
-  <si>
-    <t>-0.24 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.11 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.63 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.27 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.38 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.48 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.10 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.12 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.11 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.06 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.65 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.32 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.97 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.23 ± 0.03</t>
-  </si>
-  <si>
-    <t>-0.07 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.69 ± 0.06</t>
-  </si>
-  <si>
-    <t>0.35 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.21 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.60 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.37 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.53 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.46 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.15 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.04 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.42 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.21 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.08 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.66 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.41 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.19 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.16 ± 0.04</t>
-  </si>
-  <si>
-    <t>-9.39 ± 8.61</t>
-  </si>
-  <si>
-    <t>-0.08 ± 0.00</t>
-  </si>
-  <si>
-    <t>-1.06 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.16 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.10 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.02 ± 0.00</t>
+    <t>0.179 ± 0.009</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.014 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.65 ± 0.03</t>
+  </si>
+  <si>
+    <t>-0.05 ± 0.14</t>
+  </si>
+  <si>
+    <t>0.26 ± 0.08</t>
+  </si>
+  <si>
+    <t>0.70 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.42 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.90 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.57 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.18 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.26 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.56 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.19 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.09 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.47 ± 0.12</t>
+  </si>
+  <si>
+    <t>0.52 ± 0.06</t>
+  </si>
+  <si>
+    <t>0.88 ± 0.07</t>
+  </si>
+  <si>
+    <t>0.29 ± 0.14</t>
+  </si>
+  <si>
+    <t>0.13 ± 0.09</t>
+  </si>
+  <si>
+    <t>-0.75 ± 1.19</t>
+  </si>
+  <si>
+    <t>0.46 ± 0.01</t>
+  </si>
+  <si>
+    <t>-0.06 ± 0.09</t>
+  </si>
+  <si>
+    <t>-0.08 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.60 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.28 ± 0.15</t>
+  </si>
+  <si>
+    <t>-5.33 ± 2.93</t>
+  </si>
+  <si>
+    <t>0.50 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.16 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.04 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.45 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.30 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.43 ± 0.68</t>
+  </si>
+  <si>
+    <t>0.53 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.47 ± 0.07</t>
+  </si>
+  <si>
+    <t>0.27 ± 0.11</t>
+  </si>
+  <si>
+    <t>0.20 ± 0.07</t>
+  </si>
+  <si>
+    <t>-0.01 ± 0.07</t>
+  </si>
+  <si>
+    <t>-74.83 ± 91.96</t>
+  </si>
+  <si>
+    <t>-1.06 ± 0.06</t>
+  </si>
+  <si>
+    <t>-0.16 ± 0.02</t>
   </si>
   <si>
     <t>-0.03 ± 0.00</t>
   </si>
   <si>
+    <t>-0.03 ± 0.01</t>
+  </si>
+  <si>
     <t>-0.00 ± 0.00</t>
   </si>
   <si>
-    <t>-0.13 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.20 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.14 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.40 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.48 ± 0.00</t>
-  </si>
-  <si>
-    <t>-1.04 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.01 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.22 ± 0.00</t>
+    <t>-0.14 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.25 ± 0.03</t>
+  </si>
+  <si>
+    <t>-0.12 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.15 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.39 ± 0.06</t>
+  </si>
+  <si>
+    <t>-0.47 ± 0.03</t>
+  </si>
+  <si>
+    <t>-1.50 ± 0.54</t>
+  </si>
+  <si>
+    <t>-0.21 ± 0.02</t>
   </si>
 </sst>
 </file>
@@ -1578,7 +1593,7 @@
         <v>42</v>
       </c>
       <c r="C2">
-        <v>21.6</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1589,7 +1604,7 @@
         <v>43</v>
       </c>
       <c r="C3">
-        <v>43.2</v>
+        <v>44.1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1600,7 +1615,7 @@
         <v>44</v>
       </c>
       <c r="C4">
-        <v>28.8</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1611,7 +1626,7 @@
         <v>45</v>
       </c>
       <c r="C5">
-        <v>6.4</v>
+        <v>2.7</v>
       </c>
     </row>
   </sheetData>
@@ -1643,7 +1658,7 @@
         <v>48</v>
       </c>
       <c r="C2">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1654,7 +1669,7 @@
         <v>48</v>
       </c>
       <c r="C3">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1665,7 +1680,7 @@
         <v>48</v>
       </c>
       <c r="C4">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1712,10 +1727,10 @@
         <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1732,10 +1747,10 @@
         <v>67</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1752,10 +1767,10 @@
         <v>68</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1772,10 +1787,10 @@
         <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1792,10 +1807,10 @@
         <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1812,10 +1827,10 @@
         <v>71</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1829,13 +1844,13 @@
         <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1849,13 +1864,13 @@
         <v>64</v>
       </c>
       <c r="D9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1869,13 +1884,13 @@
         <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1893,13 +1908,13 @@
         <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1907,13 +1922,13 @@
         <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1921,13 +1936,13 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1935,13 +1950,13 @@
         <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1962,25 +1977,25 @@
         <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E1" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1991,25 +2006,25 @@
         <v>54</v>
       </c>
       <c r="C2">
-        <v>-1.04</v>
+        <v>-1.5</v>
       </c>
       <c r="D2">
         <v>-0.03</v>
       </c>
       <c r="E2">
-        <v>0.37</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F2" t="s">
         <v>13</v>
       </c>
       <c r="G2">
-        <v>0.048</v>
+        <v>0.044</v>
       </c>
       <c r="H2">
-        <v>0.0001</v>
+        <v>0.0018</v>
       </c>
       <c r="I2">
-        <v>0.0003</v>
+        <v>0.0083</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2020,25 +2035,25 @@
         <v>55</v>
       </c>
       <c r="C3">
-        <v>-9.390000000000001</v>
+        <v>-74.83</v>
       </c>
       <c r="D3">
-        <v>0.53</v>
+        <v>0.27</v>
       </c>
       <c r="E3">
-        <v>3.91</v>
+        <v>30.16</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
       </c>
       <c r="G3">
-        <v>0.043</v>
+        <v>0.037</v>
       </c>
       <c r="H3">
-        <v>0.0004</v>
+        <v>0.0063</v>
       </c>
       <c r="I3">
-        <v>0.0155</v>
+        <v>0.08649999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2049,25 +2064,25 @@
         <v>56</v>
       </c>
       <c r="C4">
-        <v>0.06</v>
+        <v>-0.75</v>
       </c>
       <c r="D4">
-        <v>0.97</v>
+        <v>0.9</v>
       </c>
       <c r="E4">
-        <v>0.37</v>
+        <v>0.61</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G4">
-        <v>0.045</v>
+        <v>0.038</v>
       </c>
       <c r="H4">
-        <v>0.0002</v>
+        <v>0.0026</v>
       </c>
       <c r="I4">
-        <v>0.0008</v>
+        <v>0.0113</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2078,10 +2093,10 @@
         <v>54</v>
       </c>
       <c r="C5">
-        <v>-0.4</v>
+        <v>-0.39</v>
       </c>
       <c r="D5">
-        <v>-0.01</v>
+        <v>-0</v>
       </c>
       <c r="E5">
         <v>0.15</v>
@@ -2090,13 +2105,13 @@
         <v>13</v>
       </c>
       <c r="G5">
-        <v>0.038</v>
+        <v>0.037</v>
       </c>
       <c r="H5">
-        <v>0.0001</v>
+        <v>0.0011</v>
       </c>
       <c r="I5">
-        <v>0.0038</v>
+        <v>0.008500000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2107,25 +2122,25 @@
         <v>55</v>
       </c>
       <c r="C6">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="D6">
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="E6">
-        <v>0.17</v>
+        <v>0.14</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
       </c>
       <c r="G6">
-        <v>0.043</v>
+        <v>0.037</v>
       </c>
       <c r="H6">
-        <v>0.0003</v>
+        <v>0.0022</v>
       </c>
       <c r="I6">
-        <v>0.0027</v>
+        <v>0.0137</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2136,25 +2151,25 @@
         <v>56</v>
       </c>
       <c r="C7">
-        <v>0.23</v>
+        <v>0.29</v>
       </c>
       <c r="D7">
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="E7">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F7" t="s">
         <v>14</v>
       </c>
       <c r="G7">
-        <v>0.041</v>
+        <v>0.033</v>
       </c>
       <c r="H7">
-        <v>0.0013</v>
+        <v>0.0028</v>
       </c>
       <c r="I7">
-        <v>0.0035</v>
+        <v>0.0132</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2180,10 +2195,10 @@
         <v>0.022</v>
       </c>
       <c r="H8">
-        <v>0.0001</v>
+        <v>0.0007</v>
       </c>
       <c r="I8">
-        <v>0.0008</v>
+        <v>0.0049</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2194,25 +2209,25 @@
         <v>55</v>
       </c>
       <c r="C9">
-        <v>-0.21</v>
+        <v>-0.06</v>
       </c>
       <c r="D9">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="E9">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
       </c>
       <c r="G9">
-        <v>0.025</v>
+        <v>0.023</v>
       </c>
       <c r="H9">
-        <v>0.0001</v>
+        <v>0.0019</v>
       </c>
       <c r="I9">
-        <v>0.0019</v>
+        <v>0.0069</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2223,10 +2238,10 @@
         <v>56</v>
       </c>
       <c r="C10">
-        <v>-0.24</v>
+        <v>-0.05</v>
       </c>
       <c r="D10">
-        <v>0.32</v>
+        <v>0.52</v>
       </c>
       <c r="E10">
         <v>0.21</v>
@@ -2235,13 +2250,13 @@
         <v>9</v>
       </c>
       <c r="G10">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="H10">
-        <v>0.0002</v>
+        <v>0.0008</v>
       </c>
       <c r="I10">
-        <v>0.0015</v>
+        <v>0.0063</v>
       </c>
     </row>
   </sheetData>
@@ -2282,10 +2297,10 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E2" t="s">
-        <v>87</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2299,10 +2314,10 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E3" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2316,10 +2331,10 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2333,10 +2348,10 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E5" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2350,10 +2365,10 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E6" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2367,10 +2382,10 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E7" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2384,10 +2399,10 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E8" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2401,10 +2416,10 @@
         <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2418,10 +2433,10 @@
         <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E10" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2435,10 +2450,10 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E11" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2452,10 +2467,10 @@
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2469,10 +2484,10 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E13" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2486,10 +2501,10 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E14" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2503,10 +2518,10 @@
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E15" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -2520,10 +2535,10 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E16" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2537,10 +2552,10 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E17" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2554,10 +2569,10 @@
         <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2571,10 +2586,10 @@
         <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E19" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2588,10 +2603,10 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E20" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2605,10 +2620,10 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E21" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2622,10 +2637,10 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>96</v>
+        <v>131</v>
       </c>
       <c r="E22" t="s">
-        <v>88</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2639,10 +2654,10 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E23" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -2656,10 +2671,10 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E24" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -2673,10 +2688,10 @@
         <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E25" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -2690,10 +2705,10 @@
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E26" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -2707,10 +2722,10 @@
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E27" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2724,10 +2739,10 @@
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E28" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2741,10 +2756,10 @@
         <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E29" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2758,10 +2773,10 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E30" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2775,10 +2790,10 @@
         <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E31" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2792,10 +2807,10 @@
         <v>13</v>
       </c>
       <c r="D32" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E32" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -2809,10 +2824,10 @@
         <v>13</v>
       </c>
       <c r="D33" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E33" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2826,10 +2841,10 @@
         <v>13</v>
       </c>
       <c r="D34" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="E34" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -2843,10 +2858,10 @@
         <v>14</v>
       </c>
       <c r="D35" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E35" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2860,10 +2875,10 @@
         <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E36" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -2877,10 +2892,10 @@
         <v>14</v>
       </c>
       <c r="D37" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E37" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2894,10 +2909,10 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E38" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2911,10 +2926,10 @@
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E39" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2928,10 +2943,10 @@
         <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E40" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -2945,10 +2960,10 @@
         <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E41" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2962,10 +2977,10 @@
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>81</v>
+        <v>150</v>
       </c>
       <c r="E42" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2979,10 +2994,10 @@
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E43" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2996,10 +3011,10 @@
         <v>11</v>
       </c>
       <c r="D44" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E44" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3013,10 +3028,10 @@
         <v>11</v>
       </c>
       <c r="D45" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E45" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -3030,10 +3045,10 @@
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E46" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -3047,10 +3062,10 @@
         <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="E47" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3064,10 +3079,10 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E48" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -3081,10 +3096,10 @@
         <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E49" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -3098,10 +3113,10 @@
         <v>13</v>
       </c>
       <c r="D50" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E50" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -3115,10 +3130,10 @@
         <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="E51" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3132,10 +3147,10 @@
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E52" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3149,10 +3164,10 @@
         <v>14</v>
       </c>
       <c r="D53" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E53" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3166,10 +3181,10 @@
         <v>14</v>
       </c>
       <c r="D54" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E54" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3183,10 +3198,10 @@
         <v>14</v>
       </c>
       <c r="D55" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E55" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace MICE/LGBM with Mean + LGBM PredOnly/Direct/Chained (fixed 300 trees); new RQs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XQmcR8UJ8WPn3HMfEePqkv
</commit_message>
<xml_diff>
--- a/results/paper/paper_assets.xlsx
+++ b/results/paper/paper_assets.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="247">
   <si>
     <t>Well</t>
   </si>
@@ -189,118 +189,145 @@
     <t>Mean</t>
   </si>
   <si>
-    <t>MICE</t>
-  </si>
-  <si>
-    <t>LGBM</t>
+    <t>LGBM-PredOnly</t>
+  </si>
+  <si>
+    <t>LGBM-Direct</t>
+  </si>
+  <si>
+    <t>LGBM-Chained</t>
   </si>
   <si>
     <t>103.8 ± 3.2</t>
   </si>
   <si>
-    <t>129.7 ± 11.2</t>
-  </si>
-  <si>
-    <t>82.7 ± 4.5</t>
+    <t>81.1 ± 4.4</t>
+  </si>
+  <si>
+    <t>81.4 ± 4.8</t>
+  </si>
+  <si>
+    <t>81.2 ± 4.1</t>
   </si>
   <si>
     <t>10.55 ± 0.07</t>
   </si>
   <si>
-    <t>6.95 ± 0.15</t>
-  </si>
-  <si>
-    <t>6.34 ± 0.19</t>
+    <t>6.40 ± 0.16</t>
+  </si>
+  <si>
+    <t>6.43 ± 0.15</t>
+  </si>
+  <si>
+    <t>6.37 ± 0.12</t>
   </si>
   <si>
     <t>0.146 ± 0.001</t>
   </si>
   <si>
-    <t>0.116 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.113 ± 0.001</t>
+    <t>0.113 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.112 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.111 ± 0.001</t>
   </si>
   <si>
     <t>26.7 ± 0.7</t>
   </si>
   <si>
-    <t>26.1 ± 1.7</t>
-  </si>
-  <si>
-    <t>13.9 ± 0.9</t>
+    <t>13.4 ± 0.8</t>
+  </si>
+  <si>
+    <t>13.5 ± 0.8</t>
+  </si>
+  <si>
+    <t>14.0 ± 0.4</t>
   </si>
   <si>
     <t>8.74 ± 0.04</t>
   </si>
   <si>
-    <t>4.99 ± 0.05</t>
-  </si>
-  <si>
-    <t>4.44 ± 0.15</t>
+    <t>4.41 ± 0.08</t>
+  </si>
+  <si>
+    <t>4.45 ± 0.09</t>
+  </si>
+  <si>
+    <t>4.36 ± 0.09</t>
   </si>
   <si>
     <t>0.117 ± 0.000</t>
   </si>
   <si>
-    <t>0.072 ± 0.001</t>
-  </si>
-  <si>
     <t>0.071 ± 0.001</t>
   </si>
   <si>
+    <t>0.070 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.068 ± 0.001</t>
+  </si>
+  <si>
     <t>0.059 ± 0.002</t>
   </si>
   <si>
-    <t>0.073 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.047 ± 0.003</t>
+    <t>0.046 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.046 ± 0.003</t>
   </si>
   <si>
     <t>0.157 ± 0.001</t>
   </si>
   <si>
-    <t>0.103 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.094 ± 0.003</t>
+    <t>0.095 ± 0.002</t>
   </si>
   <si>
     <t>0.085 ± 0.001</t>
   </si>
   <si>
-    <t>0.067 ± 0.002</t>
-  </si>
-  <si>
     <t>0.066 ± 0.001</t>
   </si>
   <si>
+    <t>0.065 ± 0.001</t>
+  </si>
+  <si>
     <t>-0.06 ± 0.00</t>
   </si>
   <si>
-    <t>-0.65 ± 0.21</t>
-  </si>
-  <si>
-    <t>0.33 ± 0.04</t>
+    <t>0.36 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.35 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.35 ± 0.03</t>
   </si>
   <si>
     <t>-0.05 ± 0.00</t>
   </si>
   <si>
-    <t>0.54 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.62 ± 0.02</t>
+    <t>0.61 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.61 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.62 ± 0.01</t>
   </si>
   <si>
     <t>-0.08 ± 0.00</t>
   </si>
   <si>
-    <t>0.32 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.35 ± 0.00</t>
+    <t>0.36 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.36 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.38 ± 0.01</t>
   </si>
   <si>
     <t>k=1</t>
@@ -315,16 +342,16 @@
     <t>0.092 ± 0.001</t>
   </si>
   <si>
-    <t>0.079 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.060 ± 0.000</t>
+    <t>0.059 ± 0.001</t>
   </si>
   <si>
     <t>0.100 ± 0.003</t>
   </si>
   <si>
-    <t>0.079 ± 0.007</t>
+    <t>0.071 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.003</t>
   </si>
   <si>
     <t>0.070 ± 0.003</t>
@@ -333,12 +360,15 @@
     <t>0.114 ± 0.003</t>
   </si>
   <si>
-    <t>0.091 ± 0.007</t>
-  </si>
-  <si>
     <t>0.078 ± 0.003</t>
   </si>
   <si>
+    <t>0.079 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.078 ± 0.002</t>
+  </si>
+  <si>
     <t>R2 wells min</t>
   </si>
   <si>
@@ -360,106 +390,145 @@
     <t>max nRMSE sd across seeds (per well)</t>
   </si>
   <si>
-    <t>0.102 ± 0.005</t>
+    <t>0.102 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.078 ± 0.012</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.051 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.013 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.142 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.103 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.075 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.117 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.089 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.007</t>
   </si>
   <si>
     <t>0.074 ± 0.005</t>
   </si>
   <si>
-    <t>0.083 ± 0.011</t>
-  </si>
-  <si>
-    <t>0.070 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.051 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.010 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.140 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.106 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.117 ± 0.001</t>
+    <t>0.039 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.001 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.153 ± 0.011</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.018 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.102 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.073 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.015</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.052 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.011 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.142 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.106 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.118 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.092 ± 0.000</t>
   </si>
   <si>
     <t>0.076 ± 0.008</t>
   </si>
   <si>
-    <t>0.074 ± 0.010</t>
-  </si>
-  <si>
-    <t>0.039 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.001 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.150 ± 0.013</t>
-  </si>
-  <si>
-    <t>0.071 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.017 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.128 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.074 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.100 ± 0.009</t>
-  </si>
-  <si>
-    <t>0.080 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.057 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.022</t>
-  </si>
-  <si>
-    <t>0.151 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.107 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.090 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.130 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.086 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.093 ± 0.018</t>
-  </si>
-  <si>
-    <t>0.070 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.041 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.159 ± 0.014</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.092 ± 0.086</t>
+    <t>0.077 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.038 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.001 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.153 ± 0.010</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.013</t>
+  </si>
+  <si>
+    <t>0.069 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.053 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.010 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.143 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.107 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.112 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.075 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.078 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.038 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.151 ± 0.015</t>
+  </si>
+  <si>
+    <t>0.011 ± 0.001</t>
   </si>
   <si>
     <t>0.180 ± 0.000</t>
@@ -474,9 +543,6 @@
     <t>0.132 ± 0.002</t>
   </si>
   <si>
-    <t>0.069 ± 0.001</t>
-  </si>
-  <si>
     <t>0.031 ± 0.001</t>
   </si>
   <si>
@@ -513,112 +579,151 @@
     <t>0.014 ± 0.001</t>
   </si>
   <si>
-    <t>0.65 ± 0.03</t>
-  </si>
-  <si>
-    <t>-0.05 ± 0.14</t>
-  </si>
-  <si>
-    <t>0.26 ± 0.08</t>
+    <t>0.65 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.03 ± 0.16</t>
+  </si>
+  <si>
+    <t>0.35 ± 0.10</t>
   </si>
   <si>
     <t>0.70 ± 0.01</t>
   </si>
   <si>
-    <t>0.42 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.90 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.57 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.18 ± 0.03</t>
+    <t>0.44 ± 0.05</t>
+  </si>
+  <si>
+    <t>0.82 ± 0.12</t>
+  </si>
+  <si>
+    <t>0.56 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.22 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.27 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.55 ± 0.05</t>
+  </si>
+  <si>
+    <t>0.25 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.10 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.47 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.53 ± 0.05</t>
+  </si>
+  <si>
+    <t>0.73 ± 0.23</t>
+  </si>
+  <si>
+    <t>0.26 ± 0.12</t>
+  </si>
+  <si>
+    <t>0.03 ± 0.07</t>
+  </si>
+  <si>
+    <t>-1.05 ± 0.84</t>
+  </si>
+  <si>
+    <t>-0.02 ± 0.09</t>
+  </si>
+  <si>
+    <t>0.34 ± 0.15</t>
+  </si>
+  <si>
+    <t>0.41 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.87 ± 0.08</t>
+  </si>
+  <si>
+    <t>0.19 ± 0.02</t>
   </si>
   <si>
     <t>0.26 ± 0.02</t>
   </si>
   <si>
-    <t>0.56 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.19 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.09 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.47 ± 0.12</t>
-  </si>
-  <si>
-    <t>0.52 ± 0.06</t>
-  </si>
-  <si>
-    <t>0.88 ± 0.07</t>
-  </si>
-  <si>
-    <t>0.29 ± 0.14</t>
-  </si>
-  <si>
-    <t>0.13 ± 0.09</t>
-  </si>
-  <si>
-    <t>-0.75 ± 1.19</t>
-  </si>
-  <si>
-    <t>0.46 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.06 ± 0.09</t>
+    <t>0.55 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.21 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.10 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.43 ± 0.08</t>
+  </si>
+  <si>
+    <t>0.56 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.68 ± 0.25</t>
+  </si>
+  <si>
+    <t>0.07 ± 0.14</t>
+  </si>
+  <si>
+    <t>-1.02 ± 0.80</t>
+  </si>
+  <si>
+    <t>0.03 ± 0.12</t>
+  </si>
+  <si>
+    <t>0.33 ± 0.10</t>
+  </si>
+  <si>
+    <t>0.70 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.40 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.88 ± 0.06</t>
+  </si>
+  <si>
+    <t>0.55 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.17 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.60 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.21 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.12 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.41 ± 0.06</t>
+  </si>
+  <si>
+    <t>0.54 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.89 ± 0.11</t>
+  </si>
+  <si>
+    <t>0.27 ± 0.15</t>
+  </si>
+  <si>
+    <t>0.12 ± 0.08</t>
+  </si>
+  <si>
+    <t>0.23 ± 0.18</t>
   </si>
   <si>
     <t>-0.08 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.60 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.28 ± 0.15</t>
-  </si>
-  <si>
-    <t>-5.33 ± 2.93</t>
-  </si>
-  <si>
-    <t>0.50 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.16 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.04 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.45 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.30 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.43 ± 0.68</t>
-  </si>
-  <si>
-    <t>0.53 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.47 ± 0.07</t>
-  </si>
-  <si>
-    <t>0.27 ± 0.11</t>
-  </si>
-  <si>
-    <t>0.20 ± 0.07</t>
-  </si>
-  <si>
-    <t>-0.01 ± 0.07</t>
-  </si>
-  <si>
-    <t>-74.83 ± 91.96</t>
   </si>
   <si>
     <t>-1.06 ± 0.06</t>
@@ -1690,7 +1795,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1721,16 +1826,16 @@
         <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="F2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1741,16 +1846,16 @@
         <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1761,36 +1866,36 @@
         <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F5" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1798,19 +1903,19 @@
         <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1818,59 +1923,59 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F7" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E9" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F9" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1878,19 +1983,79 @@
         <v>33</v>
       </c>
       <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" t="s">
+        <v>87</v>
+      </c>
+      <c r="F10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
         <v>56</v>
       </c>
-      <c r="C10" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" t="s">
-        <v>83</v>
-      </c>
-      <c r="F10" t="s">
-        <v>92</v>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" t="s">
+        <v>88</v>
+      </c>
+      <c r="F12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" t="s">
+        <v>81</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1900,7 +2065,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1908,13 +2073,13 @@
         <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="C1" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="D1" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1922,13 +2087,13 @@
         <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1936,13 +2101,13 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1950,13 +2115,27 @@
         <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="D4" t="s">
-        <v>104</v>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1966,7 +2145,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1977,25 +2156,25 @@
         <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="D1" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="E1" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="F1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="G1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="H1" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="I1" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -2035,25 +2214,25 @@
         <v>55</v>
       </c>
       <c r="C3">
-        <v>-74.83</v>
+        <v>0.12</v>
       </c>
       <c r="D3">
-        <v>0.27</v>
+        <v>0.89</v>
       </c>
       <c r="E3">
-        <v>30.16</v>
+        <v>0.35</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>0.037</v>
+        <v>0.038</v>
       </c>
       <c r="H3">
-        <v>0.0063</v>
+        <v>0.0025</v>
       </c>
       <c r="I3">
-        <v>0.08649999999999999</v>
+        <v>0.0127</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2064,54 +2243,54 @@
         <v>56</v>
       </c>
       <c r="C4">
-        <v>-0.75</v>
+        <v>-1.02</v>
       </c>
       <c r="D4">
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="E4">
-        <v>0.61</v>
+        <v>0.67</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
       </c>
       <c r="G4">
-        <v>0.038</v>
+        <v>0.037</v>
       </c>
       <c r="H4">
-        <v>0.0026</v>
+        <v>0.0027</v>
       </c>
       <c r="I4">
-        <v>0.0113</v>
+        <v>0.0153</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C5">
-        <v>-0.39</v>
+        <v>-1.05</v>
       </c>
       <c r="D5">
-        <v>-0</v>
+        <v>0.82</v>
       </c>
       <c r="E5">
-        <v>0.15</v>
+        <v>0.67</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G5">
         <v>0.037</v>
       </c>
       <c r="H5">
-        <v>0.0011</v>
+        <v>0.0023</v>
       </c>
       <c r="I5">
-        <v>0.008500000000000001</v>
+        <v>0.0122</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2119,28 +2298,28 @@
         <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6">
-        <v>0.2</v>
+        <v>-0.39</v>
       </c>
       <c r="D6">
-        <v>0.6</v>
+        <v>-0</v>
       </c>
       <c r="E6">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G6">
         <v>0.037</v>
       </c>
       <c r="H6">
-        <v>0.0022</v>
+        <v>0.0011</v>
       </c>
       <c r="I6">
-        <v>0.0137</v>
+        <v>0.008500000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2148,16 +2327,16 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7">
-        <v>0.29</v>
+        <v>0.27</v>
       </c>
       <c r="D7">
         <v>0.7</v>
       </c>
       <c r="E7">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="F7" t="s">
         <v>14</v>
@@ -2166,68 +2345,68 @@
         <v>0.033</v>
       </c>
       <c r="H7">
-        <v>0.0028</v>
+        <v>0.0024</v>
       </c>
       <c r="I7">
-        <v>0.0132</v>
+        <v>0.0153</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8">
-        <v>-1.06</v>
+        <v>0.26</v>
       </c>
       <c r="D8">
-        <v>-0</v>
+        <v>0.7</v>
       </c>
       <c r="E8">
-        <v>0.42</v>
+        <v>0.16</v>
       </c>
       <c r="F8" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G8">
-        <v>0.022</v>
+        <v>0.034</v>
       </c>
       <c r="H8">
-        <v>0.0007</v>
+        <v>0.0022</v>
       </c>
       <c r="I8">
-        <v>0.0049</v>
+        <v>0.0102</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C9">
-        <v>-0.06</v>
+        <v>0.26</v>
       </c>
       <c r="D9">
-        <v>0.47</v>
+        <v>0.7</v>
       </c>
       <c r="E9">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="F9" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G9">
-        <v>0.023</v>
+        <v>0.034</v>
       </c>
       <c r="H9">
-        <v>0.0019</v>
+        <v>0.0018</v>
       </c>
       <c r="I9">
-        <v>0.0069</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2235,28 +2414,115 @@
         <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C10">
-        <v>-0.05</v>
+        <v>-1.06</v>
       </c>
       <c r="D10">
-        <v>0.52</v>
+        <v>-0</v>
       </c>
       <c r="E10">
-        <v>0.21</v>
+        <v>0.42</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
       </c>
       <c r="G10">
+        <v>0.022</v>
+      </c>
+      <c r="H10">
+        <v>0.0007</v>
+      </c>
+      <c r="I10">
+        <v>0.0049</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11">
+        <v>0.03</v>
+      </c>
+      <c r="D11">
+        <v>0.54</v>
+      </c>
+      <c r="E11">
+        <v>0.19</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11">
         <v>0.025</v>
       </c>
-      <c r="H10">
+      <c r="H11">
+        <v>0.0014</v>
+      </c>
+      <c r="I11">
+        <v>0.0062</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12">
+        <v>-0.02</v>
+      </c>
+      <c r="D12">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E12">
+        <v>0.22</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12">
+        <v>0.025</v>
+      </c>
+      <c r="H12">
         <v>0.0008</v>
       </c>
-      <c r="I10">
-        <v>0.0063</v>
+      <c r="I12">
+        <v>0.0053</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13">
+        <v>0.03</v>
+      </c>
+      <c r="D13">
+        <v>0.53</v>
+      </c>
+      <c r="E13">
+        <v>0.2</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>0.024</v>
+      </c>
+      <c r="H13">
+        <v>0.0009</v>
+      </c>
+      <c r="I13">
+        <v>0.0056</v>
       </c>
     </row>
   </sheetData>
@@ -2266,7 +2532,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2288,7 +2554,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
         <v>32</v>
@@ -2297,15 +2563,15 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -2314,15 +2580,15 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="E3" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
         <v>31</v>
@@ -2331,15 +2597,15 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="E4" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
         <v>32</v>
@@ -2348,15 +2614,15 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
         <v>33</v>
@@ -2365,15 +2631,15 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="E6" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
@@ -2382,15 +2648,15 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="E7" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
         <v>32</v>
@@ -2399,15 +2665,15 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="E8" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
         <v>33</v>
@@ -2416,15 +2682,15 @@
         <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="E9" t="s">
-        <v>170</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
         <v>31</v>
@@ -2433,15 +2699,15 @@
         <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="E10" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
@@ -2450,15 +2716,15 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="E11" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
         <v>33</v>
@@ -2467,15 +2733,15 @@
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="E12" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B13" t="s">
         <v>31</v>
@@ -2484,15 +2750,15 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="E13" t="s">
-        <v>174</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
@@ -2501,15 +2767,15 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="E14" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
@@ -2518,15 +2784,15 @@
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E15" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
         <v>31</v>
@@ -2535,15 +2801,15 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E16" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
@@ -2552,15 +2818,15 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="E17" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
         <v>33</v>
@@ -2569,15 +2835,15 @@
         <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E18" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
         <v>31</v>
@@ -2586,15 +2852,15 @@
         <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="E19" t="s">
-        <v>180</v>
+        <v>202</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
@@ -2603,15 +2869,15 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E20" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s">
         <v>33</v>
@@ -2620,15 +2886,15 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="E21" t="s">
-        <v>182</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22" t="s">
         <v>31</v>
@@ -2637,15 +2903,15 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="E22" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B23" t="s">
         <v>32</v>
@@ -2654,15 +2920,15 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="E23" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B24" t="s">
         <v>33</v>
@@ -2671,15 +2937,15 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="E24" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
         <v>31</v>
@@ -2688,15 +2954,15 @@
         <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="E25" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
         <v>32</v>
@@ -2705,15 +2971,15 @@
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="E26" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
@@ -2722,15 +2988,15 @@
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="E27" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
         <v>31</v>
@@ -2739,15 +3005,15 @@
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E28" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B29" t="s">
         <v>32</v>
@@ -2756,15 +3022,15 @@
         <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="E29" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B30" t="s">
         <v>33</v>
@@ -2773,15 +3039,15 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="E30" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B31" t="s">
         <v>31</v>
@@ -2790,15 +3056,15 @@
         <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="E31" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B32" t="s">
         <v>32</v>
@@ -2807,15 +3073,15 @@
         <v>13</v>
       </c>
       <c r="D32" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="E32" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B33" t="s">
         <v>33</v>
@@ -2824,15 +3090,15 @@
         <v>13</v>
       </c>
       <c r="D33" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="E33" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B34" t="s">
         <v>31</v>
@@ -2841,15 +3107,15 @@
         <v>13</v>
       </c>
       <c r="D34" t="s">
-        <v>125</v>
+        <v>153</v>
       </c>
       <c r="E34" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B35" t="s">
         <v>32</v>
@@ -2858,15 +3124,15 @@
         <v>14</v>
       </c>
       <c r="D35" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="E35" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B36" t="s">
         <v>33</v>
@@ -2875,15 +3141,15 @@
         <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E36" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B37" t="s">
         <v>31</v>
@@ -2892,15 +3158,15 @@
         <v>14</v>
       </c>
       <c r="D37" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E37" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B38" t="s">
         <v>32</v>
@@ -2909,15 +3175,15 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E38" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B39" t="s">
         <v>33</v>
@@ -2926,15 +3192,15 @@
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="E39" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B40" t="s">
         <v>31</v>
@@ -2943,15 +3209,15 @@
         <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="E40" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B41" t="s">
         <v>32</v>
@@ -2960,15 +3226,15 @@
         <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="E41" t="s">
-        <v>183</v>
+        <v>219</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B42" t="s">
         <v>33</v>
@@ -2977,15 +3243,15 @@
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="E42" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B43" t="s">
         <v>31</v>
@@ -2994,15 +3260,15 @@
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="E43" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B44" t="s">
         <v>32</v>
@@ -3011,15 +3277,15 @@
         <v>11</v>
       </c>
       <c r="D44" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E44" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B45" t="s">
         <v>33</v>
@@ -3028,15 +3294,15 @@
         <v>11</v>
       </c>
       <c r="D45" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E45" t="s">
-        <v>203</v>
+        <v>223</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B46" t="s">
         <v>31</v>
@@ -3045,15 +3311,15 @@
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="E46" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B47" t="s">
         <v>32</v>
@@ -3062,15 +3328,15 @@
         <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="E47" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B48" t="s">
         <v>33</v>
@@ -3079,15 +3345,15 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>156</v>
+        <v>105</v>
       </c>
       <c r="E48" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B49" t="s">
         <v>31</v>
@@ -3096,15 +3362,15 @@
         <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="E49" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B50" t="s">
         <v>32</v>
@@ -3113,15 +3379,15 @@
         <v>13</v>
       </c>
       <c r="D50" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="E50" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B51" t="s">
         <v>33</v>
@@ -3130,15 +3396,15 @@
         <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="E51" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B52" t="s">
         <v>31</v>
@@ -3147,15 +3413,15 @@
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="E52" t="s">
-        <v>210</v>
+        <v>229</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B53" t="s">
         <v>32</v>
@@ -3164,15 +3430,15 @@
         <v>14</v>
       </c>
       <c r="D53" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="E53" t="s">
-        <v>203</v>
+        <v>230</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B54" t="s">
         <v>33</v>
@@ -3181,15 +3447,15 @@
         <v>14</v>
       </c>
       <c r="D54" t="s">
-        <v>161</v>
+        <v>109</v>
       </c>
       <c r="E54" t="s">
-        <v>203</v>
+        <v>231</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B55" t="s">
         <v>31</v>
@@ -3198,10 +3464,316 @@
         <v>14</v>
       </c>
       <c r="D55" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="E55" t="s">
-        <v>211</v>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" t="s">
+        <v>32</v>
+      </c>
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s">
+        <v>169</v>
+      </c>
+      <c r="E56" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>54</v>
+      </c>
+      <c r="B57" t="s">
+        <v>33</v>
+      </c>
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s">
+        <v>170</v>
+      </c>
+      <c r="E57" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>54</v>
+      </c>
+      <c r="B58" t="s">
+        <v>31</v>
+      </c>
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" t="s">
+        <v>171</v>
+      </c>
+      <c r="E58" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
+        <v>54</v>
+      </c>
+      <c r="B59" t="s">
+        <v>32</v>
+      </c>
+      <c r="C59" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" t="s">
+        <v>172</v>
+      </c>
+      <c r="E59" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
+        <v>54</v>
+      </c>
+      <c r="B60" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60" t="s">
+        <v>10</v>
+      </c>
+      <c r="D60" t="s">
+        <v>157</v>
+      </c>
+      <c r="E60" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>54</v>
+      </c>
+      <c r="B61" t="s">
+        <v>31</v>
+      </c>
+      <c r="C61" t="s">
+        <v>10</v>
+      </c>
+      <c r="D61" t="s">
+        <v>173</v>
+      </c>
+      <c r="E61" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" t="s">
+        <v>32</v>
+      </c>
+      <c r="C62" t="s">
+        <v>11</v>
+      </c>
+      <c r="D62" t="s">
+        <v>174</v>
+      </c>
+      <c r="E62" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" t="s">
+        <v>54</v>
+      </c>
+      <c r="B63" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" t="s">
+        <v>175</v>
+      </c>
+      <c r="E63" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
+        <v>54</v>
+      </c>
+      <c r="B64" t="s">
+        <v>31</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" t="s">
+        <v>176</v>
+      </c>
+      <c r="E64" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" t="s">
+        <v>54</v>
+      </c>
+      <c r="B65" t="s">
+        <v>32</v>
+      </c>
+      <c r="C65" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" t="s">
+        <v>177</v>
+      </c>
+      <c r="E65" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" t="s">
+        <v>54</v>
+      </c>
+      <c r="B66" t="s">
+        <v>33</v>
+      </c>
+      <c r="C66" t="s">
+        <v>12</v>
+      </c>
+      <c r="D66" t="s">
+        <v>178</v>
+      </c>
+      <c r="E66" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" t="s">
+        <v>54</v>
+      </c>
+      <c r="B67" t="s">
+        <v>31</v>
+      </c>
+      <c r="C67" t="s">
+        <v>12</v>
+      </c>
+      <c r="D67" t="s">
+        <v>179</v>
+      </c>
+      <c r="E67" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" t="s">
+        <v>54</v>
+      </c>
+      <c r="B68" t="s">
+        <v>32</v>
+      </c>
+      <c r="C68" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68" t="s">
+        <v>180</v>
+      </c>
+      <c r="E68" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" t="s">
+        <v>54</v>
+      </c>
+      <c r="B69" t="s">
+        <v>33</v>
+      </c>
+      <c r="C69" t="s">
+        <v>13</v>
+      </c>
+      <c r="D69" t="s">
+        <v>157</v>
+      </c>
+      <c r="E69" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" t="s">
+        <v>54</v>
+      </c>
+      <c r="B70" t="s">
+        <v>31</v>
+      </c>
+      <c r="C70" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" t="s">
+        <v>181</v>
+      </c>
+      <c r="E70" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" t="s">
+        <v>54</v>
+      </c>
+      <c r="B71" t="s">
+        <v>32</v>
+      </c>
+      <c r="C71" t="s">
+        <v>14</v>
+      </c>
+      <c r="D71" t="s">
+        <v>182</v>
+      </c>
+      <c r="E71" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" t="s">
+        <v>54</v>
+      </c>
+      <c r="B72" t="s">
+        <v>33</v>
+      </c>
+      <c r="C72" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72" t="s">
+        <v>183</v>
+      </c>
+      <c r="E72" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" t="s">
+        <v>54</v>
+      </c>
+      <c r="B73" t="s">
+        <v>31</v>
+      </c>
+      <c r="C73" t="s">
+        <v>14</v>
+      </c>
+      <c r="D73" t="s">
+        <v>184</v>
+      </c>
+      <c r="E73" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate results with Mean, KNN, MICE, missForest, LGBM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XQmcR8UJ8WPn3HMfEePqkv
</commit_message>
<xml_diff>
--- a/results/paper/paper_assets.xlsx
+++ b/results/paper/paper_assets.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="304">
   <si>
     <t>Well</t>
   </si>
@@ -189,580 +189,751 @@
     <t>Mean</t>
   </si>
   <si>
-    <t>LGBM-PredOnly</t>
-  </si>
-  <si>
-    <t>LGBM-Direct</t>
-  </si>
-  <si>
-    <t>LGBM-Chained</t>
+    <t>KNN</t>
+  </si>
+  <si>
+    <t>MICE</t>
+  </si>
+  <si>
+    <t>missForest</t>
+  </si>
+  <si>
+    <t>LGBM</t>
   </si>
   <si>
     <t>103.8 ± 3.2</t>
   </si>
   <si>
-    <t>81.1 ± 4.4</t>
-  </si>
-  <si>
-    <t>81.4 ± 4.8</t>
-  </si>
-  <si>
-    <t>81.2 ± 4.1</t>
+    <t>88.5 ± 4.3</t>
+  </si>
+  <si>
+    <t>129.7 ± 11.2</t>
+  </si>
+  <si>
+    <t>79.0 ± 4.1</t>
+  </si>
+  <si>
+    <t>82.7 ± 4.5</t>
   </si>
   <si>
     <t>10.55 ± 0.07</t>
   </si>
   <si>
-    <t>6.40 ± 0.16</t>
-  </si>
-  <si>
-    <t>6.43 ± 0.15</t>
-  </si>
-  <si>
-    <t>6.37 ± 0.12</t>
+    <t>6.67 ± 0.04</t>
+  </si>
+  <si>
+    <t>6.95 ± 0.15</t>
+  </si>
+  <si>
+    <t>6.33 ± 0.20</t>
+  </si>
+  <si>
+    <t>6.34 ± 0.19</t>
   </si>
   <si>
     <t>0.146 ± 0.001</t>
   </si>
   <si>
-    <t>0.113 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.112 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.111 ± 0.001</t>
+    <t>0.115 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.116 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.115 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.113 ± 0.001</t>
   </si>
   <si>
     <t>26.7 ± 0.7</t>
   </si>
   <si>
-    <t>13.4 ± 0.8</t>
-  </si>
-  <si>
-    <t>13.5 ± 0.8</t>
-  </si>
-  <si>
-    <t>14.0 ± 0.4</t>
+    <t>18.3 ± 0.8</t>
+  </si>
+  <si>
+    <t>26.1 ± 1.7</t>
+  </si>
+  <si>
+    <t>13.4 ± 0.7</t>
+  </si>
+  <si>
+    <t>13.9 ± 0.9</t>
   </si>
   <si>
     <t>8.74 ± 0.04</t>
   </si>
   <si>
-    <t>4.41 ± 0.08</t>
-  </si>
-  <si>
-    <t>4.45 ± 0.09</t>
-  </si>
-  <si>
-    <t>4.36 ± 0.09</t>
+    <t>4.47 ± 0.02</t>
+  </si>
+  <si>
+    <t>4.99 ± 0.05</t>
+  </si>
+  <si>
+    <t>4.27 ± 0.07</t>
+  </si>
+  <si>
+    <t>4.44 ± 0.15</t>
   </si>
   <si>
     <t>0.117 ± 0.000</t>
   </si>
   <si>
+    <t>0.073 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.072 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.073 ± 0.002</t>
+  </si>
+  <si>
     <t>0.071 ± 0.001</t>
   </si>
   <si>
+    <t>0.059 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.050 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.073 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.045 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.047 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.157 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.099 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.103 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.094 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.085 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.067 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.066 ± 0.001</t>
+  </si>
+  <si>
+    <t>-0.06 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.23 ± 0.03</t>
+  </si>
+  <si>
+    <t>-0.65 ± 0.21</t>
+  </si>
+  <si>
+    <t>0.39 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.33 ± 0.04</t>
+  </si>
+  <si>
+    <t>-0.05 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.58 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.54 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.62 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.08 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.33 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.32 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.35 ± 0.00</t>
+  </si>
+  <si>
+    <t>k=1</t>
+  </si>
+  <si>
+    <t>k=2</t>
+  </si>
+  <si>
+    <t>k=3</t>
+  </si>
+  <si>
+    <t>0.092 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.063 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.059 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.060 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.100 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.075 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.079 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.114 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.080 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.091 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.078 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.078 ± 0.003</t>
+  </si>
+  <si>
+    <t>R2 wells min</t>
+  </si>
+  <si>
+    <t>R2 wells max</t>
+  </si>
+  <si>
+    <t>R2 sd across wells</t>
+  </si>
+  <si>
+    <t>Worst well</t>
+  </si>
+  <si>
+    <t>nRMSE sd across wells</t>
+  </si>
+  <si>
+    <t>nRMSE sd across seeds</t>
+  </si>
+  <si>
+    <t>max nRMSE sd across seeds (per well)</t>
+  </si>
+  <si>
+    <t>0.107 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.087 ± 0.010</t>
+  </si>
+  <si>
+    <t>0.071 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.054 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.015 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.157 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.107 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.082 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.121 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.094 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.081 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.075 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.041 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.001 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.156 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.008 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.102 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.083 ± 0.011</t>
+  </si>
+  <si>
     <t>0.070 ± 0.000</t>
   </si>
   <si>
-    <t>0.068 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.059 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.046 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.046 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.157 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.095 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.085 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.066 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.065 ± 0.001</t>
-  </si>
-  <si>
-    <t>-0.06 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.36 ± 0.03</t>
+    <t>0.051 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.010 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.140 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.106 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.117 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.008</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.010</t>
+  </si>
+  <si>
+    <t>0.039 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.150 ± 0.013</t>
+  </si>
+  <si>
+    <t>0.017 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.128 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.100 ± 0.009</t>
+  </si>
+  <si>
+    <t>0.080 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.057 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.022</t>
+  </si>
+  <si>
+    <t>0.151 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.107 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.090 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.130 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.086 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.093 ± 0.018</t>
+  </si>
+  <si>
+    <t>0.041 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.159 ± 0.014</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.092 ± 0.086</t>
+  </si>
+  <si>
+    <t>0.180 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.103 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.104 ± 0.008</t>
+  </si>
+  <si>
+    <t>0.132 ± 0.002</t>
+  </si>
+  <si>
+    <t>0.069 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.031 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.217 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.117 ± 0.005</t>
+  </si>
+  <si>
+    <t>0.094 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.197 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.109 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.085 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.120 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.003 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.179 ± 0.009</t>
+  </si>
+  <si>
+    <t>0.076 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.014 ± 0.001</t>
+  </si>
+  <si>
+    <t>0.106 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.004</t>
+  </si>
+  <si>
+    <t>0.070 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.067 ± 0.000</t>
+  </si>
+  <si>
+    <t>0.016 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.142 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.113 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.088 ± 0.003</t>
+  </si>
+  <si>
+    <t>0.077 ± 0.007</t>
+  </si>
+  <si>
+    <t>0.074 ± 0.009</t>
+  </si>
+  <si>
+    <t>0.047 ± 0.006</t>
+  </si>
+  <si>
+    <t>0.158 ± 0.017</t>
+  </si>
+  <si>
+    <t>0.082 ± 0.008</t>
+  </si>
+  <si>
+    <t>0.039 ± 0.008</t>
+  </si>
+  <si>
+    <t>0.61 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.03 ± 0.05</t>
+  </si>
+  <si>
+    <t>0.18 ± 0.08</t>
+  </si>
+  <si>
+    <t>0.68 ± 0.02</t>
   </si>
   <si>
     <t>0.35 ± 0.04</t>
   </si>
   <si>
-    <t>0.35 ± 0.03</t>
-  </si>
-  <si>
-    <t>-0.05 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.61 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.61 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.62 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.08 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.36 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.36 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.38 ± 0.01</t>
-  </si>
-  <si>
-    <t>k=1</t>
-  </si>
-  <si>
-    <t>k=2</t>
-  </si>
-  <si>
-    <t>k=3</t>
-  </si>
-  <si>
-    <t>0.092 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.059 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.100 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.071 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.071 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.070 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.114 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.078 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.079 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.078 ± 0.002</t>
-  </si>
-  <si>
-    <t>R2 wells min</t>
-  </si>
-  <si>
-    <t>R2 wells max</t>
-  </si>
-  <si>
-    <t>R2 sd across wells</t>
-  </si>
-  <si>
-    <t>Worst well</t>
-  </si>
-  <si>
-    <t>nRMSE sd across wells</t>
-  </si>
-  <si>
-    <t>nRMSE sd across seeds</t>
-  </si>
-  <si>
-    <t>max nRMSE sd across seeds (per well)</t>
-  </si>
-  <si>
-    <t>0.102 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.071 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.078 ± 0.012</t>
-  </si>
-  <si>
-    <t>0.070 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.051 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.013 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.142 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.103 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.075 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.117 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.089 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.074 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.039 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.001 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.153 ± 0.011</t>
-  </si>
-  <si>
-    <t>0.074 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.018 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.102 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.073 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.079 ± 0.015</t>
-  </si>
-  <si>
-    <t>0.070 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.052 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.011 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.142 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.106 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.118 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.092 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.008</t>
-  </si>
-  <si>
-    <t>0.077 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.038 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.001 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.153 ± 0.010</t>
-  </si>
-  <si>
-    <t>0.071 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.079 ± 0.013</t>
-  </si>
-  <si>
-    <t>0.069 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.053 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.010 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.143 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.107 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.112 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.075 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.078 ± 0.006</t>
-  </si>
-  <si>
-    <t>0.038 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.151 ± 0.015</t>
-  </si>
-  <si>
-    <t>0.011 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.180 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.103 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.104 ± 0.008</t>
-  </si>
-  <si>
-    <t>0.132 ± 0.002</t>
-  </si>
-  <si>
-    <t>0.031 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.217 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.117 ± 0.005</t>
-  </si>
-  <si>
-    <t>0.094 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.197 ± 0.004</t>
-  </si>
-  <si>
-    <t>0.109 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.085 ± 0.007</t>
-  </si>
-  <si>
-    <t>0.120 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.003 ± 0.000</t>
-  </si>
-  <si>
-    <t>0.179 ± 0.009</t>
-  </si>
-  <si>
-    <t>0.076 ± 0.003</t>
-  </si>
-  <si>
-    <t>0.014 ± 0.001</t>
-  </si>
-  <si>
-    <t>0.65 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.03 ± 0.16</t>
-  </si>
-  <si>
-    <t>0.35 ± 0.10</t>
+    <t>0.77 ± 0.07</t>
+  </si>
+  <si>
+    <t>0.46 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.16 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.13 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.53 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.16 ± 0.05</t>
+  </si>
+  <si>
+    <t>-0.02 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.46 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.49 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.83 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.24 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.02 ± 0.18</t>
+  </si>
+  <si>
+    <t>0.58 ± 0.19</t>
+  </si>
+  <si>
+    <t>0.65 ± 0.03</t>
+  </si>
+  <si>
+    <t>-0.05 ± 0.14</t>
+  </si>
+  <si>
+    <t>0.26 ± 0.08</t>
   </si>
   <si>
     <t>0.70 ± 0.01</t>
   </si>
   <si>
-    <t>0.44 ± 0.05</t>
-  </si>
-  <si>
-    <t>0.82 ± 0.12</t>
+    <t>0.42 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.90 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.57 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.18 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.26 ± 0.02</t>
   </si>
   <si>
     <t>0.56 ± 0.02</t>
   </si>
   <si>
-    <t>0.22 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.27 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.55 ± 0.05</t>
-  </si>
-  <si>
-    <t>0.25 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.10 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.47 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.53 ± 0.05</t>
-  </si>
-  <si>
-    <t>0.73 ± 0.23</t>
-  </si>
-  <si>
-    <t>0.26 ± 0.12</t>
-  </si>
-  <si>
-    <t>0.03 ± 0.07</t>
-  </si>
-  <si>
-    <t>-1.05 ± 0.84</t>
-  </si>
-  <si>
-    <t>-0.02 ± 0.09</t>
-  </si>
-  <si>
-    <t>0.34 ± 0.15</t>
-  </si>
-  <si>
-    <t>0.41 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.87 ± 0.08</t>
-  </si>
-  <si>
     <t>0.19 ± 0.02</t>
   </si>
   <si>
-    <t>0.26 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.55 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.21 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.10 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.43 ± 0.08</t>
+    <t>0.09 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.47 ± 0.12</t>
+  </si>
+  <si>
+    <t>0.52 ± 0.06</t>
+  </si>
+  <si>
+    <t>0.88 ± 0.07</t>
+  </si>
+  <si>
+    <t>0.29 ± 0.14</t>
+  </si>
+  <si>
+    <t>0.13 ± 0.09</t>
+  </si>
+  <si>
+    <t>-0.75 ± 1.19</t>
+  </si>
+  <si>
+    <t>0.46 ± 0.01</t>
+  </si>
+  <si>
+    <t>-0.06 ± 0.09</t>
+  </si>
+  <si>
+    <t>-0.08 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.60 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.28 ± 0.15</t>
+  </si>
+  <si>
+    <t>-5.33 ± 2.93</t>
+  </si>
+  <si>
+    <t>0.50 ± 0.00</t>
+  </si>
+  <si>
+    <t>0.16 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.04 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.45 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.30 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.43 ± 0.68</t>
+  </si>
+  <si>
+    <t>0.53 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.47 ± 0.07</t>
+  </si>
+  <si>
+    <t>0.27 ± 0.11</t>
+  </si>
+  <si>
+    <t>0.20 ± 0.07</t>
+  </si>
+  <si>
+    <t>-0.01 ± 0.07</t>
+  </si>
+  <si>
+    <t>-74.83 ± 91.96</t>
+  </si>
+  <si>
+    <t>-1.06 ± 0.06</t>
+  </si>
+  <si>
+    <t>-0.16 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.03 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.03 ± 0.01</t>
+  </si>
+  <si>
+    <t>-0.00 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.14 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.25 ± 0.03</t>
+  </si>
+  <si>
+    <t>-0.12 ± 0.02</t>
+  </si>
+  <si>
+    <t>-0.15 ± 0.00</t>
+  </si>
+  <si>
+    <t>-0.39 ± 0.06</t>
+  </si>
+  <si>
+    <t>-0.47 ± 0.03</t>
+  </si>
+  <si>
+    <t>-1.50 ± 0.54</t>
+  </si>
+  <si>
+    <t>-0.21 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.63 ± 0.03</t>
+  </si>
+  <si>
+    <t>-0.07 ± 0.15</t>
+  </si>
+  <si>
+    <t>0.48 ± 0.04</t>
+  </si>
+  <si>
+    <t>0.72 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.42 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.73 ± 0.18</t>
   </si>
   <si>
     <t>0.56 ± 0.03</t>
   </si>
   <si>
-    <t>0.68 ± 0.25</t>
-  </si>
-  <si>
-    <t>0.07 ± 0.14</t>
-  </si>
-  <si>
-    <t>-1.02 ± 0.80</t>
-  </si>
-  <si>
-    <t>0.03 ± 0.12</t>
-  </si>
-  <si>
-    <t>0.33 ± 0.10</t>
-  </si>
-  <si>
-    <t>0.70 ± 0.00</t>
-  </si>
-  <si>
-    <t>0.40 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.88 ± 0.06</t>
-  </si>
-  <si>
-    <t>0.55 ± 0.02</t>
-  </si>
-  <si>
-    <t>0.17 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.60 ± 0.04</t>
-  </si>
-  <si>
-    <t>0.21 ± 0.01</t>
-  </si>
-  <si>
-    <t>0.12 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.41 ± 0.06</t>
-  </si>
-  <si>
-    <t>0.54 ± 0.03</t>
-  </si>
-  <si>
-    <t>0.89 ± 0.11</t>
-  </si>
-  <si>
-    <t>0.27 ± 0.15</t>
-  </si>
-  <si>
-    <t>0.12 ± 0.08</t>
-  </si>
-  <si>
-    <t>0.23 ± 0.18</t>
-  </si>
-  <si>
-    <t>-0.08 ± 0.01</t>
-  </si>
-  <si>
-    <t>-1.06 ± 0.06</t>
-  </si>
-  <si>
-    <t>-0.16 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.03 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.03 ± 0.01</t>
-  </si>
-  <si>
-    <t>-0.00 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.14 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.25 ± 0.03</t>
-  </si>
-  <si>
-    <t>-0.12 ± 0.02</t>
-  </si>
-  <si>
-    <t>-0.15 ± 0.00</t>
-  </si>
-  <si>
-    <t>-0.39 ± 0.06</t>
-  </si>
-  <si>
-    <t>-0.47 ± 0.03</t>
-  </si>
-  <si>
-    <t>-1.50 ± 0.54</t>
-  </si>
-  <si>
-    <t>-0.21 ± 0.02</t>
+    <t>0.18 ± 0.02</t>
+  </si>
+  <si>
+    <t>0.31 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.59 ± 0.03</t>
+  </si>
+  <si>
+    <t>0.26 ± 0.05</t>
+  </si>
+  <si>
+    <t>0.07 ± 0.01</t>
+  </si>
+  <si>
+    <t>0.48 ± 0.10</t>
+  </si>
+  <si>
+    <t>0.32 ± 0.15</t>
+  </si>
+  <si>
+    <t>0.89 ± 0.07</t>
+  </si>
+  <si>
+    <t>0.21 ± 0.13</t>
+  </si>
+  <si>
+    <t>-0.19 ± 0.22</t>
+  </si>
+  <si>
+    <t>-8.22 ± 2.42</t>
   </si>
 </sst>
 </file>
@@ -1795,7 +1966,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1826,16 +1997,16 @@
         <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1846,16 +2017,16 @@
         <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F3" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1866,16 +2037,16 @@
         <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="F4" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1886,36 +2057,36 @@
         <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F5" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E6" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="F6" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1923,19 +2094,19 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E7" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="F7" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1943,19 +2114,19 @@
         <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="F8" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1963,59 +2134,59 @@
         <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E9" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="F9" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E10" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F10" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="F11" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2023,19 +2194,19 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E12" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2043,19 +2214,79 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F13" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" t="s">
+        <v>86</v>
+      </c>
+      <c r="E14" t="s">
+        <v>99</v>
+      </c>
+      <c r="F14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
         <v>57</v>
       </c>
-      <c r="C13" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" t="s">
-        <v>89</v>
-      </c>
-      <c r="F13" t="s">
-        <v>101</v>
+      <c r="C15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" t="s">
+        <v>99</v>
+      </c>
+      <c r="F15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2065,7 +2296,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2073,13 +2304,13 @@
         <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="C1" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="D1" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2087,13 +2318,13 @@
         <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2101,13 +2332,13 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="D3" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2115,13 +2346,13 @@
         <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="D4" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2129,13 +2360,27 @@
         <v>57</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D6" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2145,7 +2390,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -2156,25 +2401,25 @@
         <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="D1" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="E1" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="F1" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="G1" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="H1" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="I1" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -2214,25 +2459,25 @@
         <v>55</v>
       </c>
       <c r="C3">
-        <v>0.12</v>
+        <v>-0.02</v>
       </c>
       <c r="D3">
-        <v>0.89</v>
+        <v>0.83</v>
       </c>
       <c r="E3">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
       </c>
       <c r="G3">
-        <v>0.038</v>
+        <v>0.042</v>
       </c>
       <c r="H3">
-        <v>0.0025</v>
+        <v>0.0024</v>
       </c>
       <c r="I3">
-        <v>0.0127</v>
+        <v>0.0104</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2243,13 +2488,13 @@
         <v>56</v>
       </c>
       <c r="C4">
-        <v>-1.02</v>
+        <v>-74.83</v>
       </c>
       <c r="D4">
-        <v>0.87</v>
+        <v>0.27</v>
       </c>
       <c r="E4">
-        <v>0.67</v>
+        <v>30.16</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -2258,10 +2503,10 @@
         <v>0.037</v>
       </c>
       <c r="H4">
-        <v>0.0027</v>
+        <v>0.0063</v>
       </c>
       <c r="I4">
-        <v>0.0153</v>
+        <v>0.08649999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2272,54 +2517,54 @@
         <v>57</v>
       </c>
       <c r="C5">
-        <v>-1.05</v>
+        <v>-8.220000000000001</v>
       </c>
       <c r="D5">
-        <v>0.82</v>
+        <v>0.89</v>
       </c>
       <c r="E5">
-        <v>0.67</v>
+        <v>3.57</v>
       </c>
       <c r="F5" t="s">
         <v>14</v>
       </c>
       <c r="G5">
-        <v>0.037</v>
+        <v>0.033</v>
       </c>
       <c r="H5">
         <v>0.0023</v>
       </c>
       <c r="I5">
-        <v>0.0122</v>
+        <v>0.0078</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C6">
-        <v>-0.39</v>
+        <v>-0.75</v>
       </c>
       <c r="D6">
-        <v>-0</v>
+        <v>0.9</v>
       </c>
       <c r="E6">
-        <v>0.15</v>
+        <v>0.61</v>
       </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6">
-        <v>0.037</v>
+        <v>0.038</v>
       </c>
       <c r="H6">
-        <v>0.0011</v>
+        <v>0.0026</v>
       </c>
       <c r="I6">
-        <v>0.008500000000000001</v>
+        <v>0.0113</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2327,28 +2572,28 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C7">
-        <v>0.27</v>
+        <v>-0.39</v>
       </c>
       <c r="D7">
-        <v>0.7</v>
+        <v>-0</v>
       </c>
       <c r="E7">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7">
-        <v>0.033</v>
+        <v>0.037</v>
       </c>
       <c r="H7">
-        <v>0.0024</v>
+        <v>0.0011</v>
       </c>
       <c r="I7">
-        <v>0.0153</v>
+        <v>0.008500000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2356,28 +2601,28 @@
         <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C8">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="D8">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="E8">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F8" t="s">
         <v>14</v>
       </c>
       <c r="G8">
-        <v>0.034</v>
+        <v>0.038</v>
       </c>
       <c r="H8">
-        <v>0.0022</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="I8">
-        <v>0.0102</v>
+        <v>0.0065</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2385,86 +2630,86 @@
         <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9">
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="D9">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="E9">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="F9" t="s">
         <v>14</v>
       </c>
       <c r="G9">
-        <v>0.034</v>
+        <v>0.037</v>
       </c>
       <c r="H9">
-        <v>0.0018</v>
+        <v>0.0022</v>
       </c>
       <c r="I9">
-        <v>0.011</v>
+        <v>0.0137</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C10">
-        <v>-1.06</v>
+        <v>0.21</v>
       </c>
       <c r="D10">
-        <v>-0</v>
+        <v>0.72</v>
       </c>
       <c r="E10">
-        <v>0.42</v>
+        <v>0.17</v>
       </c>
       <c r="F10" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G10">
-        <v>0.022</v>
+        <v>0.036</v>
       </c>
       <c r="H10">
-        <v>0.0007</v>
+        <v>0.003</v>
       </c>
       <c r="I10">
-        <v>0.0049</v>
+        <v>0.0174</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C11">
-        <v>0.03</v>
+        <v>0.29</v>
       </c>
       <c r="D11">
-        <v>0.54</v>
+        <v>0.7</v>
       </c>
       <c r="E11">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="F11" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G11">
-        <v>0.025</v>
+        <v>0.033</v>
       </c>
       <c r="H11">
-        <v>0.0014</v>
+        <v>0.0028</v>
       </c>
       <c r="I11">
-        <v>0.0062</v>
+        <v>0.0132</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2472,28 +2717,28 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C12">
-        <v>-0.02</v>
+        <v>-1.06</v>
       </c>
       <c r="D12">
-        <v>0.5600000000000001</v>
+        <v>-0</v>
       </c>
       <c r="E12">
-        <v>0.22</v>
+        <v>0.42</v>
       </c>
       <c r="F12" t="s">
         <v>9</v>
       </c>
       <c r="G12">
-        <v>0.025</v>
+        <v>0.022</v>
       </c>
       <c r="H12">
-        <v>0.0008</v>
+        <v>0.0007</v>
       </c>
       <c r="I12">
-        <v>0.0053</v>
+        <v>0.0049</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2501,28 +2746,115 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C13">
-        <v>0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="D13">
-        <v>0.53</v>
+        <v>0.49</v>
       </c>
       <c r="E13">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="H13">
-        <v>0.0009</v>
+        <v>0.0021</v>
       </c>
       <c r="I13">
-        <v>0.0056</v>
+        <v>0.007</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14">
+        <v>-0.06</v>
+      </c>
+      <c r="D14">
+        <v>0.47</v>
+      </c>
+      <c r="E14">
+        <v>0.2</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14">
+        <v>0.023</v>
+      </c>
+      <c r="H14">
+        <v>0.0019</v>
+      </c>
+      <c r="I14">
+        <v>0.0069</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15">
+        <v>-0.19</v>
+      </c>
+      <c r="D15">
+        <v>0.42</v>
+      </c>
+      <c r="E15">
+        <v>0.24</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15">
+        <v>0.023</v>
+      </c>
+      <c r="H15">
+        <v>0.0017</v>
+      </c>
+      <c r="I15">
+        <v>0.0076</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16">
+        <v>-0.05</v>
+      </c>
+      <c r="D16">
+        <v>0.52</v>
+      </c>
+      <c r="E16">
+        <v>0.21</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G16">
+        <v>0.025</v>
+      </c>
+      <c r="H16">
+        <v>0.0008</v>
+      </c>
+      <c r="I16">
+        <v>0.0063</v>
       </c>
     </row>
   </sheetData>
@@ -2532,7 +2864,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2554,7 +2886,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
         <v>32</v>
@@ -2563,15 +2895,15 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="E2" t="s">
-        <v>185</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -2580,15 +2912,15 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="E3" t="s">
-        <v>186</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
         <v>31</v>
@@ -2597,15 +2929,15 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="E4" t="s">
-        <v>187</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
         <v>32</v>
@@ -2614,15 +2946,15 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="E5" t="s">
-        <v>188</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
         <v>33</v>
@@ -2631,15 +2963,15 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="E6" t="s">
-        <v>189</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
@@ -2648,15 +2980,15 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>190</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
         <v>32</v>
@@ -2665,15 +2997,15 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="E8" t="s">
-        <v>191</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
         <v>33</v>
@@ -2682,15 +3014,15 @@
         <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="E9" t="s">
-        <v>192</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
         <v>31</v>
@@ -2699,15 +3031,15 @@
         <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="E10" t="s">
-        <v>193</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
@@ -2716,15 +3048,15 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="E11" t="s">
-        <v>194</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
         <v>33</v>
@@ -2733,15 +3065,15 @@
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="E12" t="s">
-        <v>195</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
         <v>31</v>
@@ -2750,15 +3082,15 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="E13" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
@@ -2767,15 +3099,15 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="E14" t="s">
-        <v>197</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
@@ -2784,15 +3116,15 @@
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="E15" t="s">
-        <v>198</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B16" t="s">
         <v>31</v>
@@ -2801,15 +3133,15 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="E16" t="s">
-        <v>199</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
@@ -2818,15 +3150,15 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="E17" t="s">
-        <v>200</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
         <v>33</v>
@@ -2835,15 +3167,15 @@
         <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="E18" t="s">
-        <v>201</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B19" t="s">
         <v>31</v>
@@ -2852,15 +3184,15 @@
         <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="E19" t="s">
-        <v>202</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
@@ -2869,15 +3201,15 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="E20" t="s">
-        <v>185</v>
+        <v>237</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B21" t="s">
         <v>33</v>
@@ -2886,15 +3218,15 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="E21" t="s">
-        <v>203</v>
+        <v>238</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B22" t="s">
         <v>31</v>
@@ -2903,15 +3235,15 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="E22" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s">
         <v>32</v>
@@ -2920,15 +3252,15 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="E23" t="s">
-        <v>188</v>
+        <v>240</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B24" t="s">
         <v>33</v>
@@ -2937,15 +3269,15 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="E24" t="s">
-        <v>205</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
         <v>31</v>
@@ -2954,15 +3286,15 @@
         <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="E25" t="s">
-        <v>206</v>
+        <v>242</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
         <v>32</v>
@@ -2971,15 +3303,15 @@
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="E26" t="s">
-        <v>191</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
@@ -2988,15 +3320,15 @@
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="E27" t="s">
-        <v>207</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B28" t="s">
         <v>31</v>
@@ -3005,15 +3337,15 @@
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>133</v>
+        <v>165</v>
       </c>
       <c r="E28" t="s">
-        <v>208</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B29" t="s">
         <v>32</v>
@@ -3022,15 +3354,15 @@
         <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="E29" t="s">
-        <v>209</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B30" t="s">
         <v>33</v>
@@ -3039,15 +3371,15 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="E30" t="s">
-        <v>210</v>
+        <v>247</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B31" t="s">
         <v>31</v>
@@ -3056,15 +3388,15 @@
         <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="E31" t="s">
-        <v>211</v>
+        <v>248</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B32" t="s">
         <v>32</v>
@@ -3073,15 +3405,15 @@
         <v>13</v>
       </c>
       <c r="D32" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="E32" t="s">
-        <v>212</v>
+        <v>249</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B33" t="s">
         <v>33</v>
@@ -3090,15 +3422,15 @@
         <v>13</v>
       </c>
       <c r="D33" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="E33" t="s">
-        <v>213</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B34" t="s">
         <v>31</v>
@@ -3110,12 +3442,12 @@
         <v>153</v>
       </c>
       <c r="E34" t="s">
-        <v>214</v>
+        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B35" t="s">
         <v>32</v>
@@ -3124,15 +3456,15 @@
         <v>14</v>
       </c>
       <c r="D35" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="E35" t="s">
-        <v>200</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B36" t="s">
         <v>33</v>
@@ -3141,15 +3473,15 @@
         <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E36" t="s">
-        <v>215</v>
+        <v>253</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B37" t="s">
         <v>31</v>
@@ -3158,15 +3490,15 @@
         <v>14</v>
       </c>
       <c r="D37" t="s">
-        <v>139</v>
+        <v>171</v>
       </c>
       <c r="E37" t="s">
-        <v>216</v>
+        <v>254</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B38" t="s">
         <v>32</v>
@@ -3175,15 +3507,15 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="E38" t="s">
-        <v>185</v>
+        <v>255</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B39" t="s">
         <v>33</v>
@@ -3192,15 +3524,15 @@
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="E39" t="s">
-        <v>217</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B40" t="s">
         <v>31</v>
@@ -3209,15 +3541,15 @@
         <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="E40" t="s">
-        <v>218</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B41" t="s">
         <v>32</v>
@@ -3226,15 +3558,15 @@
         <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="E41" t="s">
-        <v>219</v>
+        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B42" t="s">
         <v>33</v>
@@ -3243,15 +3575,15 @@
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="E42" t="s">
-        <v>220</v>
+        <v>259</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B43" t="s">
         <v>31</v>
@@ -3260,15 +3592,15 @@
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="E43" t="s">
-        <v>221</v>
+        <v>260</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B44" t="s">
         <v>32</v>
@@ -3277,15 +3609,15 @@
         <v>11</v>
       </c>
       <c r="D44" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="E44" t="s">
-        <v>222</v>
+        <v>261</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B45" t="s">
         <v>33</v>
@@ -3294,15 +3626,15 @@
         <v>11</v>
       </c>
       <c r="D45" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="E45" t="s">
-        <v>223</v>
+        <v>262</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B46" t="s">
         <v>31</v>
@@ -3311,15 +3643,15 @@
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="E46" t="s">
-        <v>195</v>
+        <v>263</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B47" t="s">
         <v>32</v>
@@ -3328,15 +3660,15 @@
         <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="E47" t="s">
-        <v>224</v>
+        <v>264</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B48" t="s">
         <v>33</v>
@@ -3345,15 +3677,15 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>105</v>
+        <v>182</v>
       </c>
       <c r="E48" t="s">
-        <v>225</v>
+        <v>265</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B49" t="s">
         <v>31</v>
@@ -3362,15 +3694,15 @@
         <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="E49" t="s">
-        <v>226</v>
+        <v>266</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B50" t="s">
         <v>32</v>
@@ -3379,15 +3711,15 @@
         <v>13</v>
       </c>
       <c r="D50" t="s">
-        <v>165</v>
+        <v>125</v>
       </c>
       <c r="E50" t="s">
-        <v>227</v>
+        <v>267</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B51" t="s">
         <v>33</v>
@@ -3396,15 +3728,15 @@
         <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="E51" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B52" t="s">
         <v>31</v>
@@ -3413,15 +3745,15 @@
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="E52" t="s">
-        <v>229</v>
+        <v>269</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B53" t="s">
         <v>32</v>
@@ -3430,15 +3762,15 @@
         <v>14</v>
       </c>
       <c r="D53" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="E53" t="s">
-        <v>230</v>
+        <v>270</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B54" t="s">
         <v>33</v>
@@ -3447,15 +3779,15 @@
         <v>14</v>
       </c>
       <c r="D54" t="s">
-        <v>109</v>
+        <v>186</v>
       </c>
       <c r="E54" t="s">
-        <v>231</v>
+        <v>271</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B55" t="s">
         <v>31</v>
@@ -3464,10 +3796,10 @@
         <v>14</v>
       </c>
       <c r="D55" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="E55" t="s">
-        <v>232</v>
+        <v>272</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -3481,10 +3813,10 @@
         <v>9</v>
       </c>
       <c r="D56" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="E56" t="s">
-        <v>233</v>
+        <v>257</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -3498,10 +3830,10 @@
         <v>9</v>
       </c>
       <c r="D57" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="E57" t="s">
-        <v>234</v>
+        <v>273</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3515,10 +3847,10 @@
         <v>9</v>
       </c>
       <c r="D58" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="E58" t="s">
-        <v>235</v>
+        <v>274</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3532,10 +3864,10 @@
         <v>10</v>
       </c>
       <c r="D59" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="E59" t="s">
-        <v>233</v>
+        <v>257</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -3549,10 +3881,10 @@
         <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="E60" t="s">
-        <v>236</v>
+        <v>275</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -3566,10 +3898,10 @@
         <v>10</v>
       </c>
       <c r="D61" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="E61" t="s">
-        <v>236</v>
+        <v>275</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3583,10 +3915,10 @@
         <v>11</v>
       </c>
       <c r="D62" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="E62" t="s">
-        <v>237</v>
+        <v>276</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3600,10 +3932,10 @@
         <v>11</v>
       </c>
       <c r="D63" t="s">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="E63" t="s">
-        <v>238</v>
+        <v>277</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3617,10 +3949,10 @@
         <v>11</v>
       </c>
       <c r="D64" t="s">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="E64" t="s">
-        <v>239</v>
+        <v>278</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3634,10 +3966,10 @@
         <v>12</v>
       </c>
       <c r="D65" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="E65" t="s">
-        <v>240</v>
+        <v>279</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3651,10 +3983,10 @@
         <v>12</v>
       </c>
       <c r="D66" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="E66" t="s">
-        <v>241</v>
+        <v>280</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3668,10 +4000,10 @@
         <v>12</v>
       </c>
       <c r="D67" t="s">
-        <v>179</v>
+        <v>199</v>
       </c>
       <c r="E67" t="s">
-        <v>242</v>
+        <v>281</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3685,10 +4017,10 @@
         <v>13</v>
       </c>
       <c r="D68" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="E68" t="s">
-        <v>243</v>
+        <v>282</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -3702,10 +4034,10 @@
         <v>13</v>
       </c>
       <c r="D69" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="E69" t="s">
-        <v>244</v>
+        <v>283</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -3719,10 +4051,10 @@
         <v>13</v>
       </c>
       <c r="D70" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="E70" t="s">
-        <v>245</v>
+        <v>284</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -3736,10 +4068,10 @@
         <v>14</v>
       </c>
       <c r="D71" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="E71" t="s">
-        <v>238</v>
+        <v>277</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3753,10 +4085,10 @@
         <v>14</v>
       </c>
       <c r="D72" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="E72" t="s">
-        <v>238</v>
+        <v>277</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3770,10 +4102,316 @@
         <v>14</v>
       </c>
       <c r="D73" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="E73" t="s">
-        <v>246</v>
+        <v>285</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" t="s">
+        <v>57</v>
+      </c>
+      <c r="B74" t="s">
+        <v>32</v>
+      </c>
+      <c r="C74" t="s">
+        <v>9</v>
+      </c>
+      <c r="D74" t="s">
+        <v>205</v>
+      </c>
+      <c r="E74" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" t="s">
+        <v>57</v>
+      </c>
+      <c r="B75" t="s">
+        <v>33</v>
+      </c>
+      <c r="C75" t="s">
+        <v>9</v>
+      </c>
+      <c r="D75" t="s">
+        <v>206</v>
+      </c>
+      <c r="E75" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" t="s">
+        <v>57</v>
+      </c>
+      <c r="B76" t="s">
+        <v>31</v>
+      </c>
+      <c r="C76" t="s">
+        <v>9</v>
+      </c>
+      <c r="D76" t="s">
+        <v>207</v>
+      </c>
+      <c r="E76" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" t="s">
+        <v>57</v>
+      </c>
+      <c r="B77" t="s">
+        <v>32</v>
+      </c>
+      <c r="C77" t="s">
+        <v>10</v>
+      </c>
+      <c r="D77" t="s">
+        <v>208</v>
+      </c>
+      <c r="E77" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" t="s">
+        <v>57</v>
+      </c>
+      <c r="B78" t="s">
+        <v>33</v>
+      </c>
+      <c r="C78" t="s">
+        <v>10</v>
+      </c>
+      <c r="D78" t="s">
+        <v>161</v>
+      </c>
+      <c r="E78" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" t="s">
+        <v>57</v>
+      </c>
+      <c r="B79" t="s">
+        <v>31</v>
+      </c>
+      <c r="C79" t="s">
+        <v>10</v>
+      </c>
+      <c r="D79" t="s">
+        <v>209</v>
+      </c>
+      <c r="E79" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80" t="s">
+        <v>57</v>
+      </c>
+      <c r="B80" t="s">
+        <v>32</v>
+      </c>
+      <c r="C80" t="s">
+        <v>11</v>
+      </c>
+      <c r="D80" t="s">
+        <v>210</v>
+      </c>
+      <c r="E80" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" t="s">
+        <v>57</v>
+      </c>
+      <c r="B81" t="s">
+        <v>33</v>
+      </c>
+      <c r="C81" t="s">
+        <v>11</v>
+      </c>
+      <c r="D81" t="s">
+        <v>205</v>
+      </c>
+      <c r="E81" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" t="s">
+        <v>57</v>
+      </c>
+      <c r="B82" t="s">
+        <v>31</v>
+      </c>
+      <c r="C82" t="s">
+        <v>11</v>
+      </c>
+      <c r="D82" t="s">
+        <v>91</v>
+      </c>
+      <c r="E82" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" t="s">
+        <v>57</v>
+      </c>
+      <c r="B83" t="s">
+        <v>32</v>
+      </c>
+      <c r="C83" t="s">
+        <v>12</v>
+      </c>
+      <c r="D83" t="s">
+        <v>211</v>
+      </c>
+      <c r="E83" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" t="s">
+        <v>57</v>
+      </c>
+      <c r="B84" t="s">
+        <v>33</v>
+      </c>
+      <c r="C84" t="s">
+        <v>12</v>
+      </c>
+      <c r="D84" t="s">
+        <v>212</v>
+      </c>
+      <c r="E84" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" t="s">
+        <v>57</v>
+      </c>
+      <c r="B85" t="s">
+        <v>31</v>
+      </c>
+      <c r="C85" t="s">
+        <v>12</v>
+      </c>
+      <c r="D85" t="s">
+        <v>213</v>
+      </c>
+      <c r="E85" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" t="s">
+        <v>57</v>
+      </c>
+      <c r="B86" t="s">
+        <v>32</v>
+      </c>
+      <c r="C86" t="s">
+        <v>13</v>
+      </c>
+      <c r="D86" t="s">
+        <v>214</v>
+      </c>
+      <c r="E86" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" t="s">
+        <v>57</v>
+      </c>
+      <c r="B87" t="s">
+        <v>33</v>
+      </c>
+      <c r="C87" t="s">
+        <v>13</v>
+      </c>
+      <c r="D87" t="s">
+        <v>215</v>
+      </c>
+      <c r="E87" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88" t="s">
+        <v>57</v>
+      </c>
+      <c r="B88" t="s">
+        <v>31</v>
+      </c>
+      <c r="C88" t="s">
+        <v>13</v>
+      </c>
+      <c r="D88" t="s">
+        <v>153</v>
+      </c>
+      <c r="E88" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89" t="s">
+        <v>57</v>
+      </c>
+      <c r="B89" t="s">
+        <v>32</v>
+      </c>
+      <c r="C89" t="s">
+        <v>14</v>
+      </c>
+      <c r="D89" t="s">
+        <v>216</v>
+      </c>
+      <c r="E89" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90" t="s">
+        <v>57</v>
+      </c>
+      <c r="B90" t="s">
+        <v>33</v>
+      </c>
+      <c r="C90" t="s">
+        <v>14</v>
+      </c>
+      <c r="D90" t="s">
+        <v>217</v>
+      </c>
+      <c r="E90" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91" t="s">
+        <v>57</v>
+      </c>
+      <c r="B91" t="s">
+        <v>31</v>
+      </c>
+      <c r="C91" t="s">
+        <v>14</v>
+      </c>
+      <c r="D91" t="s">
+        <v>218</v>
+      </c>
+      <c r="E91" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>